<commit_message>
Add styling pass and build the Dashboard sheet into the real workbook
</commit_message>
<xml_diff>
--- a/expense_tracker_2026.xlsx
+++ b/expense_tracker_2026.xlsx
@@ -7,19 +7,20 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Jan2026" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Feb2026" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Mar2026" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Apr2026" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="May2026" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Jun2026" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Jul2026" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Aug2026" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Sep2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Oct2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Nov2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Dec2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Categories" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Jan2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Feb2026" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Mar2026" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Apr2026" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="May2026" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Jun2026" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Jul2026" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Aug2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Sep2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Oct2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Nov2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Dec2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Categories" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="IncomeCategories">'Categories'!$A$3:$A$6</definedName>
@@ -42,7 +43,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +61,14 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="6">
@@ -120,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -135,6 +144,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -209,6 +224,444 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Balance Trend</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!D44</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$45:$A$56</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$D$45:$D$56</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Monthly Receipts vs Payments</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!B44</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$45:$A$56</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$B$45:$B$56</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!C44</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$45:$A$56</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$C$45:$C$56</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Spend by Main Category</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!G44</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$F$45:$F$54</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$G$45:$G$54</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Income by Source</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!J44</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$I$45:$I$48</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$J$45:$J$48</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SubCategoryDetail" displayName="SubCategoryDetail" ref="A60:C128" headerRowCount="1">
+  <autoFilter ref="A60:C128"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Main Category"/>
+    <tableColumn id="2" name="Sub-Category"/>
+    <tableColumn id="3" name="Amount"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -500,173 +953,1923 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O106"/>
+  <dimension ref="A1:M128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Site Expense Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Current Cash Balance</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>YTD Total Receipts</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>YTD Total Payments</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>Net Position (YTD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10">
+        <f>'Dec2026'!B106</f>
+        <v/>
+      </c>
+      <c r="C4" s="10">
+        <f>SUM(B45:B56)</f>
+        <v/>
+      </c>
+      <c r="E4" s="10">
+        <f>SUM(C45:C56)</f>
+        <v/>
+      </c>
+      <c r="G4" s="10">
+        <f>C4-E4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>Receipts</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>Payments</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>SNO</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Receipts</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Closing Balance</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Main Category</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>Income Category</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
         <is>
           <t>Payment Mode</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="M44" s="4" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Jan2026</t>
+        </is>
+      </c>
+      <c r="B45" s="11">
+        <f>'Jan2026'!B104</f>
+        <v/>
+      </c>
+      <c r="C45" s="11">
+        <f>'Jan2026'!B105</f>
+        <v/>
+      </c>
+      <c r="D45" s="11">
+        <f>'Jan2026'!B106</f>
+        <v/>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Land &amp; Legal</t>
+        </is>
+      </c>
+      <c r="G45" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F45)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F45)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F45)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F45)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F45)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F45)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F45)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F45)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F45)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F45)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F45)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F45)</f>
+        <v/>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Investor Capital</t>
+        </is>
+      </c>
+      <c r="J45" s="11">
+        <f>SUMIFS(Jan2026!D3:D100,Jan2026!E3:E100,$I45)+SUMIFS(Feb2026!D3:D100,Feb2026!E3:E100,$I45)+SUMIFS(Mar2026!D3:D100,Mar2026!E3:E100,$I45)+SUMIFS(Apr2026!D3:D100,Apr2026!E3:E100,$I45)+SUMIFS(May2026!D3:D100,May2026!E3:E100,$I45)+SUMIFS(Jun2026!D3:D100,Jun2026!E3:E100,$I45)+SUMIFS(Jul2026!D3:D100,Jul2026!E3:E100,$I45)+SUMIFS(Aug2026!D3:D100,Aug2026!E3:E100,$I45)+SUMIFS(Sep2026!D3:D100,Sep2026!E3:E100,$I45)+SUMIFS(Oct2026!D3:D100,Oct2026!E3:E100,$I45)+SUMIFS(Nov2026!D3:D100,Nov2026!E3:E100,$I45)+SUMIFS(Dec2026!D3:D100,Dec2026!E3:E100,$I45)</f>
+        <v/>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="M45" s="11">
+        <f>SUMIFS(Jan2026!D3:D100,Jan2026!F3:F100,$L45)+SUMIFS(Jan2026!K3:K100,Jan2026!N3:N100,$L45)+SUMIFS(Feb2026!D3:D100,Feb2026!F3:F100,$L45)+SUMIFS(Feb2026!K3:K100,Feb2026!N3:N100,$L45)+SUMIFS(Mar2026!D3:D100,Mar2026!F3:F100,$L45)+SUMIFS(Mar2026!K3:K100,Mar2026!N3:N100,$L45)+SUMIFS(Apr2026!D3:D100,Apr2026!F3:F100,$L45)+SUMIFS(Apr2026!K3:K100,Apr2026!N3:N100,$L45)+SUMIFS(May2026!D3:D100,May2026!F3:F100,$L45)+SUMIFS(May2026!K3:K100,May2026!N3:N100,$L45)+SUMIFS(Jun2026!D3:D100,Jun2026!F3:F100,$L45)+SUMIFS(Jun2026!K3:K100,Jun2026!N3:N100,$L45)+SUMIFS(Jul2026!D3:D100,Jul2026!F3:F100,$L45)+SUMIFS(Jul2026!K3:K100,Jul2026!N3:N100,$L45)+SUMIFS(Aug2026!D3:D100,Aug2026!F3:F100,$L45)+SUMIFS(Aug2026!K3:K100,Aug2026!N3:N100,$L45)+SUMIFS(Sep2026!D3:D100,Sep2026!F3:F100,$L45)+SUMIFS(Sep2026!K3:K100,Sep2026!N3:N100,$L45)+SUMIFS(Oct2026!D3:D100,Oct2026!F3:F100,$L45)+SUMIFS(Oct2026!K3:K100,Oct2026!N3:N100,$L45)+SUMIFS(Nov2026!D3:D100,Nov2026!F3:F100,$L45)+SUMIFS(Nov2026!K3:K100,Nov2026!N3:N100,$L45)+SUMIFS(Dec2026!D3:D100,Dec2026!F3:F100,$L45)+SUMIFS(Dec2026!K3:K100,Dec2026!N3:N100,$L45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Feb2026</t>
+        </is>
+      </c>
+      <c r="B46" s="11">
+        <f>'Feb2026'!B104</f>
+        <v/>
+      </c>
+      <c r="C46" s="11">
+        <f>'Feb2026'!B105</f>
+        <v/>
+      </c>
+      <c r="D46" s="11">
+        <f>'Feb2026'!B106</f>
+        <v/>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Site Development</t>
+        </is>
+      </c>
+      <c r="G46" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F46)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F46)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F46)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F46)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F46)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F46)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F46)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F46)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F46)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F46)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F46)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F46)</f>
+        <v/>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Partner Contribution</t>
+        </is>
+      </c>
+      <c r="J46" s="11">
+        <f>SUMIFS(Jan2026!D3:D100,Jan2026!E3:E100,$I46)+SUMIFS(Feb2026!D3:D100,Feb2026!E3:E100,$I46)+SUMIFS(Mar2026!D3:D100,Mar2026!E3:E100,$I46)+SUMIFS(Apr2026!D3:D100,Apr2026!E3:E100,$I46)+SUMIFS(May2026!D3:D100,May2026!E3:E100,$I46)+SUMIFS(Jun2026!D3:D100,Jun2026!E3:E100,$I46)+SUMIFS(Jul2026!D3:D100,Jul2026!E3:E100,$I46)+SUMIFS(Aug2026!D3:D100,Aug2026!E3:E100,$I46)+SUMIFS(Sep2026!D3:D100,Sep2026!E3:E100,$I46)+SUMIFS(Oct2026!D3:D100,Oct2026!E3:E100,$I46)+SUMIFS(Nov2026!D3:D100,Nov2026!E3:E100,$I46)+SUMIFS(Dec2026!D3:D100,Dec2026!E3:E100,$I46)</f>
+        <v/>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="M46" s="11">
+        <f>SUMIFS(Jan2026!D3:D100,Jan2026!F3:F100,$L46)+SUMIFS(Jan2026!K3:K100,Jan2026!N3:N100,$L46)+SUMIFS(Feb2026!D3:D100,Feb2026!F3:F100,$L46)+SUMIFS(Feb2026!K3:K100,Feb2026!N3:N100,$L46)+SUMIFS(Mar2026!D3:D100,Mar2026!F3:F100,$L46)+SUMIFS(Mar2026!K3:K100,Mar2026!N3:N100,$L46)+SUMIFS(Apr2026!D3:D100,Apr2026!F3:F100,$L46)+SUMIFS(Apr2026!K3:K100,Apr2026!N3:N100,$L46)+SUMIFS(May2026!D3:D100,May2026!F3:F100,$L46)+SUMIFS(May2026!K3:K100,May2026!N3:N100,$L46)+SUMIFS(Jun2026!D3:D100,Jun2026!F3:F100,$L46)+SUMIFS(Jun2026!K3:K100,Jun2026!N3:N100,$L46)+SUMIFS(Jul2026!D3:D100,Jul2026!F3:F100,$L46)+SUMIFS(Jul2026!K3:K100,Jul2026!N3:N100,$L46)+SUMIFS(Aug2026!D3:D100,Aug2026!F3:F100,$L46)+SUMIFS(Aug2026!K3:K100,Aug2026!N3:N100,$L46)+SUMIFS(Sep2026!D3:D100,Sep2026!F3:F100,$L46)+SUMIFS(Sep2026!K3:K100,Sep2026!N3:N100,$L46)+SUMIFS(Oct2026!D3:D100,Oct2026!F3:F100,$L46)+SUMIFS(Oct2026!K3:K100,Oct2026!N3:N100,$L46)+SUMIFS(Nov2026!D3:D100,Nov2026!F3:F100,$L46)+SUMIFS(Nov2026!K3:K100,Nov2026!N3:N100,$L46)+SUMIFS(Dec2026!D3:D100,Dec2026!F3:F100,$L46)+SUMIFS(Dec2026!K3:K100,Dec2026!N3:N100,$L46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Mar2026</t>
+        </is>
+      </c>
+      <c r="B47" s="11">
+        <f>'Mar2026'!B104</f>
+        <v/>
+      </c>
+      <c r="C47" s="11">
+        <f>'Mar2026'!B105</f>
+        <v/>
+      </c>
+      <c r="D47" s="11">
+        <f>'Mar2026'!B106</f>
+        <v/>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="G47" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F47)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F47)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F47)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F47)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F47)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F47)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F47)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F47)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F47)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F47)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F47)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F47)</f>
+        <v/>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Loan Received</t>
+        </is>
+      </c>
+      <c r="J47" s="11">
+        <f>SUMIFS(Jan2026!D3:D100,Jan2026!E3:E100,$I47)+SUMIFS(Feb2026!D3:D100,Feb2026!E3:E100,$I47)+SUMIFS(Mar2026!D3:D100,Mar2026!E3:E100,$I47)+SUMIFS(Apr2026!D3:D100,Apr2026!E3:E100,$I47)+SUMIFS(May2026!D3:D100,May2026!E3:E100,$I47)+SUMIFS(Jun2026!D3:D100,Jun2026!E3:E100,$I47)+SUMIFS(Jul2026!D3:D100,Jul2026!E3:E100,$I47)+SUMIFS(Aug2026!D3:D100,Aug2026!E3:E100,$I47)+SUMIFS(Sep2026!D3:D100,Sep2026!E3:E100,$I47)+SUMIFS(Oct2026!D3:D100,Oct2026!E3:E100,$I47)+SUMIFS(Nov2026!D3:D100,Nov2026!E3:E100,$I47)+SUMIFS(Dec2026!D3:D100,Dec2026!E3:E100,$I47)</f>
+        <v/>
+      </c>
+      <c r="M47" s="11" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Apr2026</t>
+        </is>
+      </c>
+      <c r="B48" s="11">
+        <f>'Apr2026'!B104</f>
+        <v/>
+      </c>
+      <c r="C48" s="11">
+        <f>'Apr2026'!B105</f>
+        <v/>
+      </c>
+      <c r="D48" s="11">
+        <f>'Apr2026'!B106</f>
+        <v/>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Landscaping</t>
+        </is>
+      </c>
+      <c r="G48" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F48)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F48)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F48)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F48)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F48)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F48)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F48)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F48)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F48)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F48)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F48)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F48)</f>
+        <v/>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="J48" s="11">
+        <f>SUMIFS(Jan2026!D3:D100,Jan2026!E3:E100,$I48)+SUMIFS(Feb2026!D3:D100,Feb2026!E3:E100,$I48)+SUMIFS(Mar2026!D3:D100,Mar2026!E3:E100,$I48)+SUMIFS(Apr2026!D3:D100,Apr2026!E3:E100,$I48)+SUMIFS(May2026!D3:D100,May2026!E3:E100,$I48)+SUMIFS(Jun2026!D3:D100,Jun2026!E3:E100,$I48)+SUMIFS(Jul2026!D3:D100,Jul2026!E3:E100,$I48)+SUMIFS(Aug2026!D3:D100,Aug2026!E3:E100,$I48)+SUMIFS(Sep2026!D3:D100,Sep2026!E3:E100,$I48)+SUMIFS(Oct2026!D3:D100,Oct2026!E3:E100,$I48)+SUMIFS(Nov2026!D3:D100,Nov2026!E3:E100,$I48)+SUMIFS(Dec2026!D3:D100,Dec2026!E3:E100,$I48)</f>
+        <v/>
+      </c>
+      <c r="M48" s="11" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>May2026</t>
+        </is>
+      </c>
+      <c r="B49" s="11">
+        <f>'May2026'!B104</f>
+        <v/>
+      </c>
+      <c r="C49" s="11">
+        <f>'May2026'!B105</f>
+        <v/>
+      </c>
+      <c r="D49" s="11">
+        <f>'May2026'!B106</f>
+        <v/>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Buildings &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="G49" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F49)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F49)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F49)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F49)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F49)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F49)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F49)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F49)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F49)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F49)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F49)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F49)</f>
+        <v/>
+      </c>
+      <c r="J49" s="11" t="n"/>
+      <c r="M49" s="11" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Jun2026</t>
+        </is>
+      </c>
+      <c r="B50" s="11">
+        <f>'Jun2026'!B104</f>
+        <v/>
+      </c>
+      <c r="C50" s="11">
+        <f>'Jun2026'!B105</f>
+        <v/>
+      </c>
+      <c r="D50" s="11">
+        <f>'Jun2026'!B106</f>
+        <v/>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Labour &amp; Contractors</t>
+        </is>
+      </c>
+      <c r="G50" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F50)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F50)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F50)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F50)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F50)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F50)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F50)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F50)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F50)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F50)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F50)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F50)</f>
+        <v/>
+      </c>
+      <c r="J50" s="11" t="n"/>
+      <c r="M50" s="11" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Jul2026</t>
+        </is>
+      </c>
+      <c r="B51" s="11">
+        <f>'Jul2026'!B104</f>
+        <v/>
+      </c>
+      <c r="C51" s="11">
+        <f>'Jul2026'!B105</f>
+        <v/>
+      </c>
+      <c r="D51" s="11">
+        <f>'Jul2026'!B106</f>
+        <v/>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="G51" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F51)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F51)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F51)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F51)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F51)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F51)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F51)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F51)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F51)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F51)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F51)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F51)</f>
+        <v/>
+      </c>
+      <c r="J51" s="11" t="n"/>
+      <c r="M51" s="11" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Aug2026</t>
+        </is>
+      </c>
+      <c r="B52" s="11">
+        <f>'Aug2026'!B104</f>
+        <v/>
+      </c>
+      <c r="C52" s="11">
+        <f>'Aug2026'!B105</f>
+        <v/>
+      </c>
+      <c r="D52" s="11">
+        <f>'Aug2026'!B106</f>
+        <v/>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="G52" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F52)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F52)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F52)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F52)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F52)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F52)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F52)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F52)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F52)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F52)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F52)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F52)</f>
+        <v/>
+      </c>
+      <c r="J52" s="11" t="n"/>
+      <c r="M52" s="11" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Sep2026</t>
+        </is>
+      </c>
+      <c r="B53" s="11">
+        <f>'Sep2026'!B104</f>
+        <v/>
+      </c>
+      <c r="C53" s="11">
+        <f>'Sep2026'!B105</f>
+        <v/>
+      </c>
+      <c r="D53" s="11">
+        <f>'Sep2026'!B106</f>
+        <v/>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="G53" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F53)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F53)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F53)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F53)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F53)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F53)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F53)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F53)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F53)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F53)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F53)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F53)</f>
+        <v/>
+      </c>
+      <c r="J53" s="11" t="n"/>
+      <c r="M53" s="11" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Oct2026</t>
+        </is>
+      </c>
+      <c r="B54" s="11">
+        <f>'Oct2026'!B104</f>
+        <v/>
+      </c>
+      <c r="C54" s="11">
+        <f>'Oct2026'!B105</f>
+        <v/>
+      </c>
+      <c r="D54" s="11">
+        <f>'Oct2026'!B106</f>
+        <v/>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Miscellaneous</t>
+        </is>
+      </c>
+      <c r="G54" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F54)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F54)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F54)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F54)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F54)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F54)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F54)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F54)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F54)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F54)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F54)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F54)</f>
+        <v/>
+      </c>
+      <c r="J54" s="11" t="n"/>
+      <c r="M54" s="11" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Nov2026</t>
+        </is>
+      </c>
+      <c r="B55" s="11">
+        <f>'Nov2026'!B104</f>
+        <v/>
+      </c>
+      <c r="C55" s="11">
+        <f>'Nov2026'!B105</f>
+        <v/>
+      </c>
+      <c r="D55" s="11">
+        <f>'Nov2026'!B106</f>
+        <v/>
+      </c>
+      <c r="G55" s="11" t="n"/>
+      <c r="J55" s="11" t="n"/>
+      <c r="M55" s="11" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Dec2026</t>
+        </is>
+      </c>
+      <c r="B56" s="11">
+        <f>'Dec2026'!B104</f>
+        <v/>
+      </c>
+      <c r="C56" s="11">
+        <f>'Dec2026'!B105</f>
+        <v/>
+      </c>
+      <c r="D56" s="11">
+        <f>'Dec2026'!B106</f>
+        <v/>
+      </c>
+      <c r="G56" s="11" t="n"/>
+      <c r="J56" s="11" t="n"/>
+      <c r="M56" s="11" t="n"/>
+    </row>
+    <row r="57">
+      <c r="B57" s="11" t="n"/>
+      <c r="C57" s="11" t="n"/>
+      <c r="D57" s="11" t="n"/>
+      <c r="G57" s="11" t="n"/>
+      <c r="J57" s="11" t="n"/>
+      <c r="M57" s="11" t="n"/>
+    </row>
+    <row r="58">
+      <c r="B58" s="11" t="n"/>
+      <c r="C58" s="11" t="n"/>
+      <c r="D58" s="11" t="n"/>
+      <c r="G58" s="11" t="n"/>
+      <c r="J58" s="11" t="n"/>
+      <c r="M58" s="11" t="n"/>
+    </row>
+    <row r="59">
+      <c r="B59" s="11" t="n"/>
+      <c r="C59" s="11" t="n"/>
+      <c r="D59" s="11" t="n"/>
+      <c r="G59" s="11" t="n"/>
+      <c r="J59" s="11" t="n"/>
+      <c r="M59" s="11" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
         <is>
           <t>Main Category</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="B60" s="11" t="inlineStr">
         <is>
           <t>Sub-Category</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>Payment Mode</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>Comments</t>
-        </is>
-      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="n"/>
+      <c r="G60" s="11" t="n"/>
+      <c r="J60" s="11" t="n"/>
+      <c r="M60" s="11" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Land &amp; Legal</t>
+        </is>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>Land Purchase</t>
+        </is>
+      </c>
+      <c r="C61" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A61,Jan2026!M3:M100,$B61)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A61,Feb2026!M3:M100,$B61)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A61,Mar2026!M3:M100,$B61)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A61,Apr2026!M3:M100,$B61)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A61,May2026!M3:M100,$B61)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A61,Jun2026!M3:M100,$B61)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A61,Jul2026!M3:M100,$B61)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A61,Aug2026!M3:M100,$B61)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A61,Sep2026!M3:M100,$B61)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A61,Oct2026!M3:M100,$B61)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A61,Nov2026!M3:M100,$B61)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A61,Dec2026!M3:M100,$B61)</f>
+        <v/>
+      </c>
+      <c r="D61" s="11" t="n"/>
+      <c r="G61" s="11" t="n"/>
+      <c r="J61" s="11" t="n"/>
+      <c r="M61" s="11" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Land &amp; Legal</t>
+        </is>
+      </c>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>Advance Payments</t>
+        </is>
+      </c>
+      <c r="C62" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A62,Jan2026!M3:M100,$B62)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A62,Feb2026!M3:M100,$B62)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A62,Mar2026!M3:M100,$B62)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A62,Apr2026!M3:M100,$B62)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A62,May2026!M3:M100,$B62)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A62,Jun2026!M3:M100,$B62)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A62,Jul2026!M3:M100,$B62)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A62,Aug2026!M3:M100,$B62)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A62,Sep2026!M3:M100,$B62)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A62,Oct2026!M3:M100,$B62)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A62,Nov2026!M3:M100,$B62)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A62,Dec2026!M3:M100,$B62)</f>
+        <v/>
+      </c>
+      <c r="D62" s="11" t="n"/>
+      <c r="G62" s="11" t="n"/>
+      <c r="J62" s="11" t="n"/>
+      <c r="M62" s="11" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Land &amp; Legal</t>
+        </is>
+      </c>
+      <c r="B63" s="11" t="inlineStr">
+        <is>
+          <t>Registration Charges</t>
+        </is>
+      </c>
+      <c r="C63" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A63,Jan2026!M3:M100,$B63)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A63,Feb2026!M3:M100,$B63)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A63,Mar2026!M3:M100,$B63)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A63,Apr2026!M3:M100,$B63)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A63,May2026!M3:M100,$B63)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A63,Jun2026!M3:M100,$B63)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A63,Jul2026!M3:M100,$B63)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A63,Aug2026!M3:M100,$B63)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A63,Sep2026!M3:M100,$B63)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A63,Oct2026!M3:M100,$B63)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A63,Nov2026!M3:M100,$B63)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A63,Dec2026!M3:M100,$B63)</f>
+        <v/>
+      </c>
+      <c r="D63" s="11" t="n"/>
+      <c r="G63" s="11" t="n"/>
+      <c r="J63" s="11" t="n"/>
+      <c r="M63" s="11" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Land &amp; Legal</t>
+        </is>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>Stamp Duty</t>
+        </is>
+      </c>
+      <c r="C64" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A64,Jan2026!M3:M100,$B64)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A64,Feb2026!M3:M100,$B64)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A64,Mar2026!M3:M100,$B64)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A64,Apr2026!M3:M100,$B64)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A64,May2026!M3:M100,$B64)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A64,Jun2026!M3:M100,$B64)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A64,Jul2026!M3:M100,$B64)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A64,Aug2026!M3:M100,$B64)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A64,Sep2026!M3:M100,$B64)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A64,Oct2026!M3:M100,$B64)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A64,Nov2026!M3:M100,$B64)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A64,Dec2026!M3:M100,$B64)</f>
+        <v/>
+      </c>
+      <c r="D64" s="11" t="n"/>
+      <c r="G64" s="11" t="n"/>
+      <c r="J64" s="11" t="n"/>
+      <c r="M64" s="11" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Land &amp; Legal</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>Legal Fees</t>
+        </is>
+      </c>
+      <c r="C65" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A65,Jan2026!M3:M100,$B65)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A65,Feb2026!M3:M100,$B65)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A65,Mar2026!M3:M100,$B65)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A65,Apr2026!M3:M100,$B65)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A65,May2026!M3:M100,$B65)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A65,Jun2026!M3:M100,$B65)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A65,Jul2026!M3:M100,$B65)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A65,Aug2026!M3:M100,$B65)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A65,Sep2026!M3:M100,$B65)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A65,Oct2026!M3:M100,$B65)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A65,Nov2026!M3:M100,$B65)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A65,Dec2026!M3:M100,$B65)</f>
+        <v/>
+      </c>
+      <c r="D65" s="11" t="n"/>
+      <c r="G65" s="11" t="n"/>
+      <c r="J65" s="11" t="n"/>
+      <c r="M65" s="11" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Land &amp; Legal</t>
+        </is>
+      </c>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>Survey Charges</t>
+        </is>
+      </c>
+      <c r="C66" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A66,Jan2026!M3:M100,$B66)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A66,Feb2026!M3:M100,$B66)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A66,Mar2026!M3:M100,$B66)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A66,Apr2026!M3:M100,$B66)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A66,May2026!M3:M100,$B66)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A66,Jun2026!M3:M100,$B66)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A66,Jul2026!M3:M100,$B66)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A66,Aug2026!M3:M100,$B66)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A66,Sep2026!M3:M100,$B66)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A66,Oct2026!M3:M100,$B66)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A66,Nov2026!M3:M100,$B66)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A66,Dec2026!M3:M100,$B66)</f>
+        <v/>
+      </c>
+      <c r="D66" s="11" t="n"/>
+      <c r="G66" s="11" t="n"/>
+      <c r="J66" s="11" t="n"/>
+      <c r="M66" s="11" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Land &amp; Legal</t>
+        </is>
+      </c>
+      <c r="B67" s="11" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="C67" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A67,Jan2026!M3:M100,$B67)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A67,Feb2026!M3:M100,$B67)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A67,Mar2026!M3:M100,$B67)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A67,Apr2026!M3:M100,$B67)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A67,May2026!M3:M100,$B67)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A67,Jun2026!M3:M100,$B67)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A67,Jul2026!M3:M100,$B67)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A67,Aug2026!M3:M100,$B67)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A67,Sep2026!M3:M100,$B67)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A67,Oct2026!M3:M100,$B67)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A67,Nov2026!M3:M100,$B67)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A67,Dec2026!M3:M100,$B67)</f>
+        <v/>
+      </c>
+      <c r="D67" s="11" t="n"/>
+      <c r="G67" s="11" t="n"/>
+      <c r="J67" s="11" t="n"/>
+      <c r="M67" s="11" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Site Development</t>
+        </is>
+      </c>
+      <c r="B68" s="11" t="inlineStr">
+        <is>
+          <t>Land Clearing</t>
+        </is>
+      </c>
+      <c r="C68" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A68,Jan2026!M3:M100,$B68)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A68,Feb2026!M3:M100,$B68)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A68,Mar2026!M3:M100,$B68)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A68,Apr2026!M3:M100,$B68)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A68,May2026!M3:M100,$B68)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A68,Jun2026!M3:M100,$B68)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A68,Jul2026!M3:M100,$B68)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A68,Aug2026!M3:M100,$B68)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A68,Sep2026!M3:M100,$B68)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A68,Oct2026!M3:M100,$B68)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A68,Nov2026!M3:M100,$B68)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A68,Dec2026!M3:M100,$B68)</f>
+        <v/>
+      </c>
+      <c r="D68" s="11" t="n"/>
+      <c r="G68" s="11" t="n"/>
+      <c r="J68" s="11" t="n"/>
+      <c r="M68" s="11" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Site Development</t>
+        </is>
+      </c>
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>Earthwork &amp; Levelling</t>
+        </is>
+      </c>
+      <c r="C69" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A69,Jan2026!M3:M100,$B69)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A69,Feb2026!M3:M100,$B69)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A69,Mar2026!M3:M100,$B69)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A69,Apr2026!M3:M100,$B69)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A69,May2026!M3:M100,$B69)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A69,Jun2026!M3:M100,$B69)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A69,Jul2026!M3:M100,$B69)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A69,Aug2026!M3:M100,$B69)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A69,Sep2026!M3:M100,$B69)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A69,Oct2026!M3:M100,$B69)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A69,Nov2026!M3:M100,$B69)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A69,Dec2026!M3:M100,$B69)</f>
+        <v/>
+      </c>
+      <c r="D69" s="11" t="n"/>
+      <c r="G69" s="11" t="n"/>
+      <c r="J69" s="11" t="n"/>
+      <c r="M69" s="11" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Site Development</t>
+        </is>
+      </c>
+      <c r="B70" s="11" t="inlineStr">
+        <is>
+          <t>Road Formation</t>
+        </is>
+      </c>
+      <c r="C70" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A70,Jan2026!M3:M100,$B70)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A70,Feb2026!M3:M100,$B70)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A70,Mar2026!M3:M100,$B70)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A70,Apr2026!M3:M100,$B70)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A70,May2026!M3:M100,$B70)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A70,Jun2026!M3:M100,$B70)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A70,Jul2026!M3:M100,$B70)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A70,Aug2026!M3:M100,$B70)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A70,Sep2026!M3:M100,$B70)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A70,Oct2026!M3:M100,$B70)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A70,Nov2026!M3:M100,$B70)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A70,Dec2026!M3:M100,$B70)</f>
+        <v/>
+      </c>
+      <c r="D70" s="11" t="n"/>
+      <c r="G70" s="11" t="n"/>
+      <c r="J70" s="11" t="n"/>
+      <c r="M70" s="11" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Site Development</t>
+        </is>
+      </c>
+      <c r="B71" s="11" t="inlineStr">
+        <is>
+          <t>Blacktop Roads</t>
+        </is>
+      </c>
+      <c r="C71" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A71,Jan2026!M3:M100,$B71)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A71,Feb2026!M3:M100,$B71)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A71,Mar2026!M3:M100,$B71)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A71,Apr2026!M3:M100,$B71)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A71,May2026!M3:M100,$B71)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A71,Jun2026!M3:M100,$B71)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A71,Jul2026!M3:M100,$B71)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A71,Aug2026!M3:M100,$B71)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A71,Sep2026!M3:M100,$B71)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A71,Oct2026!M3:M100,$B71)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A71,Nov2026!M3:M100,$B71)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A71,Dec2026!M3:M100,$B71)</f>
+        <v/>
+      </c>
+      <c r="D71" s="11" t="n"/>
+      <c r="G71" s="11" t="n"/>
+      <c r="J71" s="11" t="n"/>
+      <c r="M71" s="11" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Site Development</t>
+        </is>
+      </c>
+      <c r="B72" s="11" t="inlineStr">
+        <is>
+          <t>Interlocking Pavers</t>
+        </is>
+      </c>
+      <c r="C72" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A72,Jan2026!M3:M100,$B72)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A72,Feb2026!M3:M100,$B72)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A72,Mar2026!M3:M100,$B72)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A72,Apr2026!M3:M100,$B72)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A72,May2026!M3:M100,$B72)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A72,Jun2026!M3:M100,$B72)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A72,Jul2026!M3:M100,$B72)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A72,Aug2026!M3:M100,$B72)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A72,Sep2026!M3:M100,$B72)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A72,Oct2026!M3:M100,$B72)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A72,Nov2026!M3:M100,$B72)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A72,Dec2026!M3:M100,$B72)</f>
+        <v/>
+      </c>
+      <c r="D72" s="11" t="n"/>
+      <c r="G72" s="11" t="n"/>
+      <c r="J72" s="11" t="n"/>
+      <c r="M72" s="11" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Site Development</t>
+        </is>
+      </c>
+      <c r="B73" s="11" t="inlineStr">
+        <is>
+          <t>Compound Wall</t>
+        </is>
+      </c>
+      <c r="C73" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A73,Jan2026!M3:M100,$B73)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A73,Feb2026!M3:M100,$B73)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A73,Mar2026!M3:M100,$B73)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A73,Apr2026!M3:M100,$B73)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A73,May2026!M3:M100,$B73)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A73,Jun2026!M3:M100,$B73)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A73,Jul2026!M3:M100,$B73)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A73,Aug2026!M3:M100,$B73)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A73,Sep2026!M3:M100,$B73)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A73,Oct2026!M3:M100,$B73)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A73,Nov2026!M3:M100,$B73)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A73,Dec2026!M3:M100,$B73)</f>
+        <v/>
+      </c>
+      <c r="D73" s="11" t="n"/>
+      <c r="G73" s="11" t="n"/>
+      <c r="J73" s="11" t="n"/>
+      <c r="M73" s="11" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Site Development</t>
+        </is>
+      </c>
+      <c r="B74" s="11" t="inlineStr">
+        <is>
+          <t>Entrance Gate</t>
+        </is>
+      </c>
+      <c r="C74" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A74,Jan2026!M3:M100,$B74)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A74,Feb2026!M3:M100,$B74)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A74,Mar2026!M3:M100,$B74)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A74,Apr2026!M3:M100,$B74)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A74,May2026!M3:M100,$B74)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A74,Jun2026!M3:M100,$B74)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A74,Jul2026!M3:M100,$B74)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A74,Aug2026!M3:M100,$B74)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A74,Sep2026!M3:M100,$B74)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A74,Oct2026!M3:M100,$B74)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A74,Nov2026!M3:M100,$B74)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A74,Dec2026!M3:M100,$B74)</f>
+        <v/>
+      </c>
+      <c r="D74" s="11" t="n"/>
+      <c r="G74" s="11" t="n"/>
+      <c r="J74" s="11" t="n"/>
+      <c r="M74" s="11" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Site Development</t>
+        </is>
+      </c>
+      <c r="B75" s="11" t="inlineStr">
+        <is>
+          <t>Drainage</t>
+        </is>
+      </c>
+      <c r="C75" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A75,Jan2026!M3:M100,$B75)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A75,Feb2026!M3:M100,$B75)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A75,Mar2026!M3:M100,$B75)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A75,Apr2026!M3:M100,$B75)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A75,May2026!M3:M100,$B75)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A75,Jun2026!M3:M100,$B75)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A75,Jul2026!M3:M100,$B75)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A75,Aug2026!M3:M100,$B75)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A75,Sep2026!M3:M100,$B75)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A75,Oct2026!M3:M100,$B75)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A75,Nov2026!M3:M100,$B75)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A75,Dec2026!M3:M100,$B75)</f>
+        <v/>
+      </c>
+      <c r="D75" s="11" t="n"/>
+      <c r="G75" s="11" t="n"/>
+      <c r="J75" s="11" t="n"/>
+      <c r="M75" s="11" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Site Development</t>
+        </is>
+      </c>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>Culverts</t>
+        </is>
+      </c>
+      <c r="C76" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A76,Jan2026!M3:M100,$B76)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A76,Feb2026!M3:M100,$B76)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A76,Mar2026!M3:M100,$B76)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A76,Apr2026!M3:M100,$B76)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A76,May2026!M3:M100,$B76)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A76,Jun2026!M3:M100,$B76)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A76,Jul2026!M3:M100,$B76)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A76,Aug2026!M3:M100,$B76)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A76,Sep2026!M3:M100,$B76)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A76,Oct2026!M3:M100,$B76)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A76,Nov2026!M3:M100,$B76)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A76,Dec2026!M3:M100,$B76)</f>
+        <v/>
+      </c>
+      <c r="D76" s="11" t="n"/>
+      <c r="G76" s="11" t="n"/>
+      <c r="J76" s="11" t="n"/>
+      <c r="M76" s="11" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>Borewell</t>
+        </is>
+      </c>
+      <c r="C77" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A77,Jan2026!M3:M100,$B77)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A77,Feb2026!M3:M100,$B77)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A77,Mar2026!M3:M100,$B77)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A77,Apr2026!M3:M100,$B77)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A77,May2026!M3:M100,$B77)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A77,Jun2026!M3:M100,$B77)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A77,Jul2026!M3:M100,$B77)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A77,Aug2026!M3:M100,$B77)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A77,Sep2026!M3:M100,$B77)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A77,Oct2026!M3:M100,$B77)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A77,Nov2026!M3:M100,$B77)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A77,Dec2026!M3:M100,$B77)</f>
+        <v/>
+      </c>
+      <c r="D77" s="11" t="n"/>
+      <c r="G77" s="11" t="n"/>
+      <c r="J77" s="11" t="n"/>
+      <c r="M77" s="11" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>Water Pipelines</t>
+        </is>
+      </c>
+      <c r="C78" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A78,Jan2026!M3:M100,$B78)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A78,Feb2026!M3:M100,$B78)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A78,Mar2026!M3:M100,$B78)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A78,Apr2026!M3:M100,$B78)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A78,May2026!M3:M100,$B78)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A78,Jun2026!M3:M100,$B78)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A78,Jul2026!M3:M100,$B78)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A78,Aug2026!M3:M100,$B78)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A78,Sep2026!M3:M100,$B78)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A78,Oct2026!M3:M100,$B78)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A78,Nov2026!M3:M100,$B78)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A78,Dec2026!M3:M100,$B78)</f>
+        <v/>
+      </c>
+      <c r="D78" s="11" t="n"/>
+      <c r="G78" s="11" t="n"/>
+      <c r="J78" s="11" t="n"/>
+      <c r="M78" s="11" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="B79" s="11" t="inlineStr">
+        <is>
+          <t>Water Tank</t>
+        </is>
+      </c>
+      <c r="C79" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A79,Jan2026!M3:M100,$B79)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A79,Feb2026!M3:M100,$B79)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A79,Mar2026!M3:M100,$B79)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A79,Apr2026!M3:M100,$B79)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A79,May2026!M3:M100,$B79)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A79,Jun2026!M3:M100,$B79)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A79,Jul2026!M3:M100,$B79)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A79,Aug2026!M3:M100,$B79)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A79,Sep2026!M3:M100,$B79)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A79,Oct2026!M3:M100,$B79)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A79,Nov2026!M3:M100,$B79)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A79,Dec2026!M3:M100,$B79)</f>
+        <v/>
+      </c>
+      <c r="D79" s="11" t="n"/>
+      <c r="G79" s="11" t="n"/>
+      <c r="J79" s="11" t="n"/>
+      <c r="M79" s="11" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="B80" s="11" t="inlineStr">
+        <is>
+          <t>Electricity Connection</t>
+        </is>
+      </c>
+      <c r="C80" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A80,Jan2026!M3:M100,$B80)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A80,Feb2026!M3:M100,$B80)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A80,Mar2026!M3:M100,$B80)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A80,Apr2026!M3:M100,$B80)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A80,May2026!M3:M100,$B80)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A80,Jun2026!M3:M100,$B80)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A80,Jul2026!M3:M100,$B80)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A80,Aug2026!M3:M100,$B80)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A80,Sep2026!M3:M100,$B80)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A80,Oct2026!M3:M100,$B80)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A80,Nov2026!M3:M100,$B80)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A80,Dec2026!M3:M100,$B80)</f>
+        <v/>
+      </c>
+      <c r="D80" s="11" t="n"/>
+      <c r="G80" s="11" t="n"/>
+      <c r="J80" s="11" t="n"/>
+      <c r="M80" s="11" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="B81" s="11" t="inlineStr">
+        <is>
+          <t>Transformer</t>
+        </is>
+      </c>
+      <c r="C81" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A81,Jan2026!M3:M100,$B81)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A81,Feb2026!M3:M100,$B81)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A81,Mar2026!M3:M100,$B81)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A81,Apr2026!M3:M100,$B81)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A81,May2026!M3:M100,$B81)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A81,Jun2026!M3:M100,$B81)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A81,Jul2026!M3:M100,$B81)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A81,Aug2026!M3:M100,$B81)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A81,Sep2026!M3:M100,$B81)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A81,Oct2026!M3:M100,$B81)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A81,Nov2026!M3:M100,$B81)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A81,Dec2026!M3:M100,$B81)</f>
+        <v/>
+      </c>
+      <c r="D81" s="11" t="n"/>
+      <c r="G81" s="11" t="n"/>
+      <c r="J81" s="11" t="n"/>
+      <c r="M81" s="11" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="B82" s="11" t="inlineStr">
+        <is>
+          <t>Street Lights</t>
+        </is>
+      </c>
+      <c r="C82" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A82,Jan2026!M3:M100,$B82)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A82,Feb2026!M3:M100,$B82)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A82,Mar2026!M3:M100,$B82)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A82,Apr2026!M3:M100,$B82)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A82,May2026!M3:M100,$B82)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A82,Jun2026!M3:M100,$B82)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A82,Jul2026!M3:M100,$B82)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A82,Aug2026!M3:M100,$B82)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A82,Sep2026!M3:M100,$B82)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A82,Oct2026!M3:M100,$B82)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A82,Nov2026!M3:M100,$B82)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A82,Dec2026!M3:M100,$B82)</f>
+        <v/>
+      </c>
+      <c r="D82" s="11" t="n"/>
+      <c r="G82" s="11" t="n"/>
+      <c r="J82" s="11" t="n"/>
+      <c r="M82" s="11" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="B83" s="11" t="inlineStr">
+        <is>
+          <t>Generator</t>
+        </is>
+      </c>
+      <c r="C83" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A83,Jan2026!M3:M100,$B83)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A83,Feb2026!M3:M100,$B83)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A83,Mar2026!M3:M100,$B83)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A83,Apr2026!M3:M100,$B83)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A83,May2026!M3:M100,$B83)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A83,Jun2026!M3:M100,$B83)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A83,Jul2026!M3:M100,$B83)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A83,Aug2026!M3:M100,$B83)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A83,Sep2026!M3:M100,$B83)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A83,Oct2026!M3:M100,$B83)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A83,Nov2026!M3:M100,$B83)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A83,Dec2026!M3:M100,$B83)</f>
+        <v/>
+      </c>
+      <c r="D83" s="11" t="n"/>
+      <c r="G83" s="11" t="n"/>
+      <c r="J83" s="11" t="n"/>
+      <c r="M83" s="11" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Landscaping</t>
+        </is>
+      </c>
+      <c r="B84" s="11" t="inlineStr">
+        <is>
+          <t>Plantation</t>
+        </is>
+      </c>
+      <c r="C84" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A84,Jan2026!M3:M100,$B84)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A84,Feb2026!M3:M100,$B84)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A84,Mar2026!M3:M100,$B84)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A84,Apr2026!M3:M100,$B84)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A84,May2026!M3:M100,$B84)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A84,Jun2026!M3:M100,$B84)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A84,Jul2026!M3:M100,$B84)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A84,Aug2026!M3:M100,$B84)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A84,Sep2026!M3:M100,$B84)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A84,Oct2026!M3:M100,$B84)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A84,Nov2026!M3:M100,$B84)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A84,Dec2026!M3:M100,$B84)</f>
+        <v/>
+      </c>
+      <c r="D84" s="11" t="n"/>
+      <c r="G84" s="11" t="n"/>
+      <c r="J84" s="11" t="n"/>
+      <c r="M84" s="11" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Landscaping</t>
+        </is>
+      </c>
+      <c r="B85" s="11" t="inlineStr">
+        <is>
+          <t>Miyawaki Forest</t>
+        </is>
+      </c>
+      <c r="C85" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A85,Jan2026!M3:M100,$B85)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A85,Feb2026!M3:M100,$B85)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A85,Mar2026!M3:M100,$B85)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A85,Apr2026!M3:M100,$B85)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A85,May2026!M3:M100,$B85)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A85,Jun2026!M3:M100,$B85)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A85,Jul2026!M3:M100,$B85)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A85,Aug2026!M3:M100,$B85)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A85,Sep2026!M3:M100,$B85)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A85,Oct2026!M3:M100,$B85)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A85,Nov2026!M3:M100,$B85)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A85,Dec2026!M3:M100,$B85)</f>
+        <v/>
+      </c>
+      <c r="D85" s="11" t="n"/>
+      <c r="G85" s="11" t="n"/>
+      <c r="J85" s="11" t="n"/>
+      <c r="M85" s="11" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Landscaping</t>
+        </is>
+      </c>
+      <c r="B86" s="11" t="inlineStr">
+        <is>
+          <t>Lawn Development</t>
+        </is>
+      </c>
+      <c r="C86" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A86,Jan2026!M3:M100,$B86)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A86,Feb2026!M3:M100,$B86)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A86,Mar2026!M3:M100,$B86)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A86,Apr2026!M3:M100,$B86)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A86,May2026!M3:M100,$B86)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A86,Jun2026!M3:M100,$B86)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A86,Jul2026!M3:M100,$B86)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A86,Aug2026!M3:M100,$B86)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A86,Sep2026!M3:M100,$B86)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A86,Oct2026!M3:M100,$B86)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A86,Nov2026!M3:M100,$B86)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A86,Dec2026!M3:M100,$B86)</f>
+        <v/>
+      </c>
+      <c r="D86" s="11" t="n"/>
+      <c r="G86" s="11" t="n"/>
+      <c r="J86" s="11" t="n"/>
+      <c r="M86" s="11" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Landscaping</t>
+        </is>
+      </c>
+      <c r="B87" s="11" t="inlineStr">
+        <is>
+          <t>Irrigation/Drip System</t>
+        </is>
+      </c>
+      <c r="C87" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A87,Jan2026!M3:M100,$B87)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A87,Feb2026!M3:M100,$B87)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A87,Mar2026!M3:M100,$B87)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A87,Apr2026!M3:M100,$B87)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A87,May2026!M3:M100,$B87)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A87,Jun2026!M3:M100,$B87)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A87,Jul2026!M3:M100,$B87)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A87,Aug2026!M3:M100,$B87)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A87,Sep2026!M3:M100,$B87)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A87,Oct2026!M3:M100,$B87)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A87,Nov2026!M3:M100,$B87)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A87,Dec2026!M3:M100,$B87)</f>
+        <v/>
+      </c>
+      <c r="D87" s="11" t="n"/>
+      <c r="G87" s="11" t="n"/>
+      <c r="J87" s="11" t="n"/>
+      <c r="M87" s="11" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Landscaping</t>
+        </is>
+      </c>
+      <c r="B88" s="11" t="inlineStr">
+        <is>
+          <t>Garden Maintenance</t>
+        </is>
+      </c>
+      <c r="C88" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A88,Jan2026!M3:M100,$B88)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A88,Feb2026!M3:M100,$B88)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A88,Mar2026!M3:M100,$B88)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A88,Apr2026!M3:M100,$B88)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A88,May2026!M3:M100,$B88)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A88,Jun2026!M3:M100,$B88)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A88,Jul2026!M3:M100,$B88)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A88,Aug2026!M3:M100,$B88)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A88,Sep2026!M3:M100,$B88)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A88,Oct2026!M3:M100,$B88)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A88,Nov2026!M3:M100,$B88)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A88,Dec2026!M3:M100,$B88)</f>
+        <v/>
+      </c>
+      <c r="D88" s="11" t="n"/>
+      <c r="G88" s="11" t="n"/>
+      <c r="J88" s="11" t="n"/>
+      <c r="M88" s="11" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Buildings &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="B89" s="11" t="inlineStr">
+        <is>
+          <t>Security Room</t>
+        </is>
+      </c>
+      <c r="C89" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A89,Jan2026!M3:M100,$B89)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A89,Feb2026!M3:M100,$B89)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A89,Mar2026!M3:M100,$B89)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A89,Apr2026!M3:M100,$B89)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A89,May2026!M3:M100,$B89)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A89,Jun2026!M3:M100,$B89)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A89,Jul2026!M3:M100,$B89)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A89,Aug2026!M3:M100,$B89)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A89,Sep2026!M3:M100,$B89)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A89,Oct2026!M3:M100,$B89)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A89,Nov2026!M3:M100,$B89)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A89,Dec2026!M3:M100,$B89)</f>
+        <v/>
+      </c>
+      <c r="D89" s="11" t="n"/>
+      <c r="G89" s="11" t="n"/>
+      <c r="J89" s="11" t="n"/>
+      <c r="M89" s="11" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Buildings &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="B90" s="11" t="inlineStr">
+        <is>
+          <t>Site Office</t>
+        </is>
+      </c>
+      <c r="C90" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A90,Jan2026!M3:M100,$B90)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A90,Feb2026!M3:M100,$B90)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A90,Mar2026!M3:M100,$B90)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A90,Apr2026!M3:M100,$B90)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A90,May2026!M3:M100,$B90)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A90,Jun2026!M3:M100,$B90)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A90,Jul2026!M3:M100,$B90)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A90,Aug2026!M3:M100,$B90)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A90,Sep2026!M3:M100,$B90)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A90,Oct2026!M3:M100,$B90)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A90,Nov2026!M3:M100,$B90)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A90,Dec2026!M3:M100,$B90)</f>
+        <v/>
+      </c>
+      <c r="D90" s="11" t="n"/>
+      <c r="G90" s="11" t="n"/>
+      <c r="J90" s="11" t="n"/>
+      <c r="M90" s="11" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Buildings &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="B91" s="11" t="inlineStr">
+        <is>
+          <t>Clubhouse</t>
+        </is>
+      </c>
+      <c r="C91" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A91,Jan2026!M3:M100,$B91)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A91,Feb2026!M3:M100,$B91)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A91,Mar2026!M3:M100,$B91)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A91,Apr2026!M3:M100,$B91)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A91,May2026!M3:M100,$B91)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A91,Jun2026!M3:M100,$B91)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A91,Jul2026!M3:M100,$B91)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A91,Aug2026!M3:M100,$B91)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A91,Sep2026!M3:M100,$B91)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A91,Oct2026!M3:M100,$B91)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A91,Nov2026!M3:M100,$B91)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A91,Dec2026!M3:M100,$B91)</f>
+        <v/>
+      </c>
+      <c r="D91" s="11" t="n"/>
+      <c r="G91" s="11" t="n"/>
+      <c r="J91" s="11" t="n"/>
+      <c r="M91" s="11" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Buildings &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="B92" s="11" t="inlineStr">
+        <is>
+          <t>Swimming Pool</t>
+        </is>
+      </c>
+      <c r="C92" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A92,Jan2026!M3:M100,$B92)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A92,Feb2026!M3:M100,$B92)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A92,Mar2026!M3:M100,$B92)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A92,Apr2026!M3:M100,$B92)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A92,May2026!M3:M100,$B92)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A92,Jun2026!M3:M100,$B92)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A92,Jul2026!M3:M100,$B92)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A92,Aug2026!M3:M100,$B92)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A92,Sep2026!M3:M100,$B92)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A92,Oct2026!M3:M100,$B92)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A92,Nov2026!M3:M100,$B92)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A92,Dec2026!M3:M100,$B92)</f>
+        <v/>
+      </c>
+      <c r="D92" s="11" t="n"/>
+      <c r="G92" s="11" t="n"/>
+      <c r="J92" s="11" t="n"/>
+      <c r="M92" s="11" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Buildings &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="B93" s="11" t="inlineStr">
+        <is>
+          <t>Gazebo</t>
+        </is>
+      </c>
+      <c r="C93" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A93,Jan2026!M3:M100,$B93)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A93,Feb2026!M3:M100,$B93)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A93,Mar2026!M3:M100,$B93)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A93,Apr2026!M3:M100,$B93)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A93,May2026!M3:M100,$B93)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A93,Jun2026!M3:M100,$B93)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A93,Jul2026!M3:M100,$B93)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A93,Aug2026!M3:M100,$B93)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A93,Sep2026!M3:M100,$B93)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A93,Oct2026!M3:M100,$B93)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A93,Nov2026!M3:M100,$B93)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A93,Dec2026!M3:M100,$B93)</f>
+        <v/>
+      </c>
+      <c r="D93" s="11" t="n"/>
+      <c r="G93" s="11" t="n"/>
+      <c r="J93" s="11" t="n"/>
+      <c r="M93" s="11" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Buildings &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="B94" s="11" t="inlineStr">
+        <is>
+          <t>Children's Play Area</t>
+        </is>
+      </c>
+      <c r="C94" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A94,Jan2026!M3:M100,$B94)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A94,Feb2026!M3:M100,$B94)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A94,Mar2026!M3:M100,$B94)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A94,Apr2026!M3:M100,$B94)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A94,May2026!M3:M100,$B94)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A94,Jun2026!M3:M100,$B94)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A94,Jul2026!M3:M100,$B94)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A94,Aug2026!M3:M100,$B94)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A94,Sep2026!M3:M100,$B94)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A94,Oct2026!M3:M100,$B94)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A94,Nov2026!M3:M100,$B94)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A94,Dec2026!M3:M100,$B94)</f>
+        <v/>
+      </c>
+      <c r="D94" s="11" t="n"/>
+      <c r="G94" s="11" t="n"/>
+      <c r="J94" s="11" t="n"/>
+      <c r="M94" s="11" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Buildings &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="B95" s="11" t="inlineStr">
+        <is>
+          <t>Sports Courts</t>
+        </is>
+      </c>
+      <c r="C95" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A95,Jan2026!M3:M100,$B95)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A95,Feb2026!M3:M100,$B95)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A95,Mar2026!M3:M100,$B95)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A95,Apr2026!M3:M100,$B95)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A95,May2026!M3:M100,$B95)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A95,Jun2026!M3:M100,$B95)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A95,Jul2026!M3:M100,$B95)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A95,Aug2026!M3:M100,$B95)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A95,Sep2026!M3:M100,$B95)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A95,Oct2026!M3:M100,$B95)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A95,Nov2026!M3:M100,$B95)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A95,Dec2026!M3:M100,$B95)</f>
+        <v/>
+      </c>
+      <c r="D95" s="11" t="n"/>
+      <c r="G95" s="11" t="n"/>
+      <c r="J95" s="11" t="n"/>
+      <c r="M95" s="11" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Buildings &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="B96" s="11" t="inlineStr">
+        <is>
+          <t>Toilets</t>
+        </is>
+      </c>
+      <c r="C96" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A96,Jan2026!M3:M100,$B96)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A96,Feb2026!M3:M100,$B96)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A96,Mar2026!M3:M100,$B96)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A96,Apr2026!M3:M100,$B96)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A96,May2026!M3:M100,$B96)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A96,Jun2026!M3:M100,$B96)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A96,Jul2026!M3:M100,$B96)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A96,Aug2026!M3:M100,$B96)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A96,Sep2026!M3:M100,$B96)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A96,Oct2026!M3:M100,$B96)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A96,Nov2026!M3:M100,$B96)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A96,Dec2026!M3:M100,$B96)</f>
+        <v/>
+      </c>
+      <c r="D96" s="11" t="n"/>
+      <c r="G96" s="11" t="n"/>
+      <c r="J96" s="11" t="n"/>
+      <c r="M96" s="11" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Labour &amp; Contractors</t>
+        </is>
+      </c>
+      <c r="B97" s="11" t="inlineStr">
+        <is>
+          <t>Labour Wages</t>
+        </is>
+      </c>
+      <c r="C97" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A97,Jan2026!M3:M100,$B97)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A97,Feb2026!M3:M100,$B97)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A97,Mar2026!M3:M100,$B97)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A97,Apr2026!M3:M100,$B97)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A97,May2026!M3:M100,$B97)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A97,Jun2026!M3:M100,$B97)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A97,Jul2026!M3:M100,$B97)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A97,Aug2026!M3:M100,$B97)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A97,Sep2026!M3:M100,$B97)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A97,Oct2026!M3:M100,$B97)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A97,Nov2026!M3:M100,$B97)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A97,Dec2026!M3:M100,$B97)</f>
+        <v/>
+      </c>
+      <c r="D97" s="11" t="n"/>
+      <c r="G97" s="11" t="n"/>
+      <c r="J97" s="11" t="n"/>
+      <c r="M97" s="11" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Labour &amp; Contractors</t>
+        </is>
+      </c>
+      <c r="B98" s="11" t="inlineStr">
+        <is>
+          <t>Contractor Payments</t>
+        </is>
+      </c>
+      <c r="C98" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A98,Jan2026!M3:M100,$B98)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A98,Feb2026!M3:M100,$B98)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A98,Mar2026!M3:M100,$B98)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A98,Apr2026!M3:M100,$B98)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A98,May2026!M3:M100,$B98)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A98,Jun2026!M3:M100,$B98)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A98,Jul2026!M3:M100,$B98)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A98,Aug2026!M3:M100,$B98)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A98,Sep2026!M3:M100,$B98)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A98,Oct2026!M3:M100,$B98)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A98,Nov2026!M3:M100,$B98)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A98,Dec2026!M3:M100,$B98)</f>
+        <v/>
+      </c>
+      <c r="D98" s="11" t="n"/>
+      <c r="G98" s="11" t="n"/>
+      <c r="J98" s="11" t="n"/>
+      <c r="M98" s="11" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Labour &amp; Contractors</t>
+        </is>
+      </c>
+      <c r="B99" s="11" t="inlineStr">
+        <is>
+          <t>Machinery Hire</t>
+        </is>
+      </c>
+      <c r="C99" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A99,Jan2026!M3:M100,$B99)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A99,Feb2026!M3:M100,$B99)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A99,Mar2026!M3:M100,$B99)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A99,Apr2026!M3:M100,$B99)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A99,May2026!M3:M100,$B99)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A99,Jun2026!M3:M100,$B99)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A99,Jul2026!M3:M100,$B99)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A99,Aug2026!M3:M100,$B99)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A99,Sep2026!M3:M100,$B99)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A99,Oct2026!M3:M100,$B99)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A99,Nov2026!M3:M100,$B99)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A99,Dec2026!M3:M100,$B99)</f>
+        <v/>
+      </c>
+      <c r="D99" s="11" t="n"/>
+      <c r="G99" s="11" t="n"/>
+      <c r="J99" s="11" t="n"/>
+      <c r="M99" s="11" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Labour &amp; Contractors</t>
+        </is>
+      </c>
+      <c r="B100" s="11" t="inlineStr">
+        <is>
+          <t>Excavator/JCB</t>
+        </is>
+      </c>
+      <c r="C100" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A100,Jan2026!M3:M100,$B100)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A100,Feb2026!M3:M100,$B100)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A100,Mar2026!M3:M100,$B100)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A100,Apr2026!M3:M100,$B100)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A100,May2026!M3:M100,$B100)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A100,Jun2026!M3:M100,$B100)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A100,Jul2026!M3:M100,$B100)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A100,Aug2026!M3:M100,$B100)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A100,Sep2026!M3:M100,$B100)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A100,Oct2026!M3:M100,$B100)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A100,Nov2026!M3:M100,$B100)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A100,Dec2026!M3:M100,$B100)</f>
+        <v/>
+      </c>
+      <c r="D100" s="11" t="n"/>
+      <c r="G100" s="11" t="n"/>
+      <c r="J100" s="11" t="n"/>
+      <c r="M100" s="11" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Labour &amp; Contractors</t>
+        </is>
+      </c>
+      <c r="B101" s="11" t="inlineStr">
+        <is>
+          <t>Tractor &amp; Transport</t>
+        </is>
+      </c>
+      <c r="C101" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A101,Jan2026!M3:M100,$B101)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A101,Feb2026!M3:M100,$B101)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A101,Mar2026!M3:M100,$B101)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A101,Apr2026!M3:M100,$B101)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A101,May2026!M3:M100,$B101)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A101,Jun2026!M3:M100,$B101)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A101,Jul2026!M3:M100,$B101)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A101,Aug2026!M3:M100,$B101)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A101,Sep2026!M3:M100,$B101)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A101,Oct2026!M3:M100,$B101)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A101,Nov2026!M3:M100,$B101)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A101,Dec2026!M3:M100,$B101)</f>
+        <v/>
+      </c>
+      <c r="D101" s="11" t="n"/>
+      <c r="G101" s="11" t="n"/>
+      <c r="J101" s="11" t="n"/>
+      <c r="M101" s="11" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="B102" s="11" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="C102" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A102,Jan2026!M3:M100,$B102)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A102,Feb2026!M3:M100,$B102)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A102,Mar2026!M3:M100,$B102)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A102,Apr2026!M3:M100,$B102)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A102,May2026!M3:M100,$B102)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A102,Jun2026!M3:M100,$B102)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A102,Jul2026!M3:M100,$B102)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A102,Aug2026!M3:M100,$B102)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A102,Sep2026!M3:M100,$B102)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A102,Oct2026!M3:M100,$B102)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A102,Nov2026!M3:M100,$B102)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A102,Dec2026!M3:M100,$B102)</f>
+        <v/>
+      </c>
+      <c r="D102" s="11" t="n"/>
+      <c r="G102" s="11" t="n"/>
+      <c r="J102" s="11" t="n"/>
+      <c r="M102" s="11" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="6" t="inlineStr">
-        <is>
-          <t>Opening Balance</t>
-        </is>
-      </c>
-      <c r="B103" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="B103" s="11" t="inlineStr">
+        <is>
+          <t>Sand</t>
+        </is>
+      </c>
+      <c r="C103" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A103,Jan2026!M3:M100,$B103)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A103,Feb2026!M3:M100,$B103)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A103,Mar2026!M3:M100,$B103)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A103,Apr2026!M3:M100,$B103)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A103,May2026!M3:M100,$B103)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A103,Jun2026!M3:M100,$B103)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A103,Jul2026!M3:M100,$B103)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A103,Aug2026!M3:M100,$B103)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A103,Sep2026!M3:M100,$B103)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A103,Oct2026!M3:M100,$B103)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A103,Nov2026!M3:M100,$B103)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A103,Dec2026!M3:M100,$B103)</f>
+        <v/>
+      </c>
+      <c r="D103" s="11" t="n"/>
+      <c r="G103" s="11" t="n"/>
+      <c r="J103" s="11" t="n"/>
+      <c r="M103" s="11" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="6" t="inlineStr">
-        <is>
-          <t>Total Receipts</t>
-        </is>
-      </c>
-      <c r="B104" s="7">
-        <f>SUM(D3:D100)</f>
-        <v/>
-      </c>
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="B104" s="11" t="inlineStr">
+        <is>
+          <t>Metal</t>
+        </is>
+      </c>
+      <c r="C104" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A104,Jan2026!M3:M100,$B104)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A104,Feb2026!M3:M100,$B104)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A104,Mar2026!M3:M100,$B104)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A104,Apr2026!M3:M100,$B104)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A104,May2026!M3:M100,$B104)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A104,Jun2026!M3:M100,$B104)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A104,Jul2026!M3:M100,$B104)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A104,Aug2026!M3:M100,$B104)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A104,Sep2026!M3:M100,$B104)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A104,Oct2026!M3:M100,$B104)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A104,Nov2026!M3:M100,$B104)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A104,Dec2026!M3:M100,$B104)</f>
+        <v/>
+      </c>
+      <c r="D104" s="11" t="n"/>
+      <c r="G104" s="11" t="n"/>
+      <c r="J104" s="11" t="n"/>
+      <c r="M104" s="11" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="6" t="inlineStr">
-        <is>
-          <t>Total Payments</t>
-        </is>
-      </c>
-      <c r="B105" s="7">
-        <f>SUM(K3:K100)</f>
-        <v/>
-      </c>
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="B105" s="11" t="inlineStr">
+        <is>
+          <t>Bricks</t>
+        </is>
+      </c>
+      <c r="C105" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A105,Jan2026!M3:M100,$B105)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A105,Feb2026!M3:M100,$B105)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A105,Mar2026!M3:M100,$B105)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A105,Apr2026!M3:M100,$B105)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A105,May2026!M3:M100,$B105)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A105,Jun2026!M3:M100,$B105)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A105,Jul2026!M3:M100,$B105)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A105,Aug2026!M3:M100,$B105)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A105,Sep2026!M3:M100,$B105)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A105,Oct2026!M3:M100,$B105)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A105,Nov2026!M3:M100,$B105)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A105,Dec2026!M3:M100,$B105)</f>
+        <v/>
+      </c>
+      <c r="D105" s="11" t="n"/>
+      <c r="G105" s="11" t="n"/>
+      <c r="J105" s="11" t="n"/>
+      <c r="M105" s="11" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="6" t="inlineStr">
-        <is>
-          <t>Net / Closing Balance</t>
-        </is>
-      </c>
-      <c r="B106" s="7">
-        <f>B103+B104-B105</f>
-        <v/>
-      </c>
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="B106" s="11" t="inlineStr">
+        <is>
+          <t>Steel</t>
+        </is>
+      </c>
+      <c r="C106" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A106,Jan2026!M3:M100,$B106)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A106,Feb2026!M3:M100,$B106)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A106,Mar2026!M3:M100,$B106)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A106,Apr2026!M3:M100,$B106)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A106,May2026!M3:M100,$B106)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A106,Jun2026!M3:M100,$B106)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A106,Jul2026!M3:M100,$B106)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A106,Aug2026!M3:M100,$B106)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A106,Sep2026!M3:M100,$B106)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A106,Oct2026!M3:M100,$B106)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A106,Nov2026!M3:M100,$B106)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A106,Dec2026!M3:M100,$B106)</f>
+        <v/>
+      </c>
+      <c r="D106" s="11" t="n"/>
+      <c r="G106" s="11" t="n"/>
+      <c r="J106" s="11" t="n"/>
+      <c r="M106" s="11" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="B107" s="11" t="inlineStr">
+        <is>
+          <t>Pipes</t>
+        </is>
+      </c>
+      <c r="C107" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A107,Jan2026!M3:M100,$B107)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A107,Feb2026!M3:M100,$B107)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A107,Mar2026!M3:M100,$B107)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A107,Apr2026!M3:M100,$B107)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A107,May2026!M3:M100,$B107)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A107,Jun2026!M3:M100,$B107)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A107,Jul2026!M3:M100,$B107)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A107,Aug2026!M3:M100,$B107)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A107,Sep2026!M3:M100,$B107)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A107,Oct2026!M3:M100,$B107)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A107,Nov2026!M3:M100,$B107)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A107,Dec2026!M3:M100,$B107)</f>
+        <v/>
+      </c>
+      <c r="D107" s="11" t="n"/>
+      <c r="G107" s="11" t="n"/>
+      <c r="J107" s="11" t="n"/>
+      <c r="M107" s="11" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="B108" s="11" t="inlineStr">
+        <is>
+          <t>Electrical Materials</t>
+        </is>
+      </c>
+      <c r="C108" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A108,Jan2026!M3:M100,$B108)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A108,Feb2026!M3:M100,$B108)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A108,Mar2026!M3:M100,$B108)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A108,Apr2026!M3:M100,$B108)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A108,May2026!M3:M100,$B108)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A108,Jun2026!M3:M100,$B108)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A108,Jul2026!M3:M100,$B108)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A108,Aug2026!M3:M100,$B108)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A108,Sep2026!M3:M100,$B108)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A108,Oct2026!M3:M100,$B108)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A108,Nov2026!M3:M100,$B108)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A108,Dec2026!M3:M100,$B108)</f>
+        <v/>
+      </c>
+      <c r="D108" s="11" t="n"/>
+      <c r="G108" s="11" t="n"/>
+      <c r="J108" s="11" t="n"/>
+      <c r="M108" s="11" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="B109" s="11" t="inlineStr">
+        <is>
+          <t>Paint</t>
+        </is>
+      </c>
+      <c r="C109" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A109,Jan2026!M3:M100,$B109)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A109,Feb2026!M3:M100,$B109)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A109,Mar2026!M3:M100,$B109)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A109,Apr2026!M3:M100,$B109)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A109,May2026!M3:M100,$B109)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A109,Jun2026!M3:M100,$B109)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A109,Jul2026!M3:M100,$B109)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A109,Aug2026!M3:M100,$B109)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A109,Sep2026!M3:M100,$B109)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A109,Oct2026!M3:M100,$B109)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A109,Nov2026!M3:M100,$B109)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A109,Dec2026!M3:M100,$B109)</f>
+        <v/>
+      </c>
+      <c r="D109" s="11" t="n"/>
+      <c r="G109" s="11" t="n"/>
+      <c r="J109" s="11" t="n"/>
+      <c r="M109" s="11" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="B110" s="11" t="inlineStr">
+        <is>
+          <t>Tiles</t>
+        </is>
+      </c>
+      <c r="C110" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A110,Jan2026!M3:M100,$B110)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A110,Feb2026!M3:M100,$B110)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A110,Mar2026!M3:M100,$B110)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A110,Apr2026!M3:M100,$B110)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A110,May2026!M3:M100,$B110)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A110,Jun2026!M3:M100,$B110)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A110,Jul2026!M3:M100,$B110)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A110,Aug2026!M3:M100,$B110)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A110,Sep2026!M3:M100,$B110)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A110,Oct2026!M3:M100,$B110)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A110,Nov2026!M3:M100,$B110)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A110,Dec2026!M3:M100,$B110)</f>
+        <v/>
+      </c>
+      <c r="D110" s="11" t="n"/>
+      <c r="G110" s="11" t="n"/>
+      <c r="J110" s="11" t="n"/>
+      <c r="M110" s="11" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="B111" s="11" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C111" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A111,Jan2026!M3:M100,$B111)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A111,Feb2026!M3:M100,$B111)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A111,Mar2026!M3:M100,$B111)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A111,Apr2026!M3:M100,$B111)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A111,May2026!M3:M100,$B111)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A111,Jun2026!M3:M100,$B111)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A111,Jul2026!M3:M100,$B111)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A111,Aug2026!M3:M100,$B111)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A111,Sep2026!M3:M100,$B111)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A111,Oct2026!M3:M100,$B111)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A111,Nov2026!M3:M100,$B111)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A111,Dec2026!M3:M100,$B111)</f>
+        <v/>
+      </c>
+      <c r="D111" s="11" t="n"/>
+      <c r="G111" s="11" t="n"/>
+      <c r="J111" s="11" t="n"/>
+      <c r="M111" s="11" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="B112" s="11" t="inlineStr">
+        <is>
+          <t>Housekeeping</t>
+        </is>
+      </c>
+      <c r="C112" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A112,Jan2026!M3:M100,$B112)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A112,Feb2026!M3:M100,$B112)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A112,Mar2026!M3:M100,$B112)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A112,Apr2026!M3:M100,$B112)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A112,May2026!M3:M100,$B112)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A112,Jun2026!M3:M100,$B112)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A112,Jul2026!M3:M100,$B112)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A112,Aug2026!M3:M100,$B112)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A112,Sep2026!M3:M100,$B112)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A112,Oct2026!M3:M100,$B112)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A112,Nov2026!M3:M100,$B112)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A112,Dec2026!M3:M100,$B112)</f>
+        <v/>
+      </c>
+      <c r="D112" s="11" t="n"/>
+      <c r="G112" s="11" t="n"/>
+      <c r="J112" s="11" t="n"/>
+      <c r="M112" s="11" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="B113" s="11" t="inlineStr">
+        <is>
+          <t>Fuel &amp; Diesel</t>
+        </is>
+      </c>
+      <c r="C113" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A113,Jan2026!M3:M100,$B113)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A113,Feb2026!M3:M100,$B113)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A113,Mar2026!M3:M100,$B113)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A113,Apr2026!M3:M100,$B113)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A113,May2026!M3:M100,$B113)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A113,Jun2026!M3:M100,$B113)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A113,Jul2026!M3:M100,$B113)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A113,Aug2026!M3:M100,$B113)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A113,Sep2026!M3:M100,$B113)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A113,Oct2026!M3:M100,$B113)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A113,Nov2026!M3:M100,$B113)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A113,Dec2026!M3:M100,$B113)</f>
+        <v/>
+      </c>
+      <c r="D113" s="11" t="n"/>
+      <c r="G113" s="11" t="n"/>
+      <c r="J113" s="11" t="n"/>
+      <c r="M113" s="11" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="B114" s="11" t="inlineStr">
+        <is>
+          <t>Vehicle Expenses</t>
+        </is>
+      </c>
+      <c r="C114" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A114,Jan2026!M3:M100,$B114)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A114,Feb2026!M3:M100,$B114)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A114,Mar2026!M3:M100,$B114)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A114,Apr2026!M3:M100,$B114)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A114,May2026!M3:M100,$B114)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A114,Jun2026!M3:M100,$B114)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A114,Jul2026!M3:M100,$B114)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A114,Aug2026!M3:M100,$B114)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A114,Sep2026!M3:M100,$B114)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A114,Oct2026!M3:M100,$B114)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A114,Nov2026!M3:M100,$B114)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A114,Dec2026!M3:M100,$B114)</f>
+        <v/>
+      </c>
+      <c r="D114" s="11" t="n"/>
+      <c r="G114" s="11" t="n"/>
+      <c r="J114" s="11" t="n"/>
+      <c r="M114" s="11" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="B115" s="11" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="C115" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A115,Jan2026!M3:M100,$B115)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A115,Feb2026!M3:M100,$B115)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A115,Mar2026!M3:M100,$B115)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A115,Apr2026!M3:M100,$B115)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A115,May2026!M3:M100,$B115)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A115,Jun2026!M3:M100,$B115)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A115,Jul2026!M3:M100,$B115)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A115,Aug2026!M3:M100,$B115)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A115,Sep2026!M3:M100,$B115)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A115,Oct2026!M3:M100,$B115)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A115,Nov2026!M3:M100,$B115)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A115,Dec2026!M3:M100,$B115)</f>
+        <v/>
+      </c>
+      <c r="D115" s="11" t="n"/>
+      <c r="G115" s="11" t="n"/>
+      <c r="J115" s="11" t="n"/>
+      <c r="M115" s="11" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="B116" s="11" t="inlineStr">
+        <is>
+          <t>Office Expenses</t>
+        </is>
+      </c>
+      <c r="C116" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A116,Jan2026!M3:M100,$B116)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A116,Feb2026!M3:M100,$B116)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A116,Mar2026!M3:M100,$B116)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A116,Apr2026!M3:M100,$B116)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A116,May2026!M3:M100,$B116)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A116,Jun2026!M3:M100,$B116)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A116,Jul2026!M3:M100,$B116)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A116,Aug2026!M3:M100,$B116)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A116,Sep2026!M3:M100,$B116)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A116,Oct2026!M3:M100,$B116)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A116,Nov2026!M3:M100,$B116)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A116,Dec2026!M3:M100,$B116)</f>
+        <v/>
+      </c>
+      <c r="D116" s="11" t="n"/>
+      <c r="G116" s="11" t="n"/>
+      <c r="J116" s="11" t="n"/>
+      <c r="M116" s="11" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="B117" s="11" t="inlineStr">
+        <is>
+          <t>Internet &amp; Phone</t>
+        </is>
+      </c>
+      <c r="C117" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A117,Jan2026!M3:M100,$B117)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A117,Feb2026!M3:M100,$B117)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A117,Mar2026!M3:M100,$B117)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A117,Apr2026!M3:M100,$B117)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A117,May2026!M3:M100,$B117)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A117,Jun2026!M3:M100,$B117)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A117,Jul2026!M3:M100,$B117)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A117,Aug2026!M3:M100,$B117)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A117,Sep2026!M3:M100,$B117)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A117,Oct2026!M3:M100,$B117)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A117,Nov2026!M3:M100,$B117)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A117,Dec2026!M3:M100,$B117)</f>
+        <v/>
+      </c>
+      <c r="D117" s="11" t="n"/>
+      <c r="G117" s="11" t="n"/>
+      <c r="J117" s="11" t="n"/>
+      <c r="M117" s="11" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="B118" s="11" t="inlineStr">
+        <is>
+          <t>Advertisement</t>
+        </is>
+      </c>
+      <c r="C118" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A118,Jan2026!M3:M100,$B118)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A118,Feb2026!M3:M100,$B118)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A118,Mar2026!M3:M100,$B118)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A118,Apr2026!M3:M100,$B118)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A118,May2026!M3:M100,$B118)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A118,Jun2026!M3:M100,$B118)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A118,Jul2026!M3:M100,$B118)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A118,Aug2026!M3:M100,$B118)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A118,Sep2026!M3:M100,$B118)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A118,Oct2026!M3:M100,$B118)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A118,Nov2026!M3:M100,$B118)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A118,Dec2026!M3:M100,$B118)</f>
+        <v/>
+      </c>
+      <c r="D118" s="11" t="n"/>
+      <c r="G118" s="11" t="n"/>
+      <c r="J118" s="11" t="n"/>
+      <c r="M118" s="11" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="B119" s="11" t="inlineStr">
+        <is>
+          <t>Flex Boards</t>
+        </is>
+      </c>
+      <c r="C119" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A119,Jan2026!M3:M100,$B119)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A119,Feb2026!M3:M100,$B119)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A119,Mar2026!M3:M100,$B119)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A119,Apr2026!M3:M100,$B119)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A119,May2026!M3:M100,$B119)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A119,Jun2026!M3:M100,$B119)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A119,Jul2026!M3:M100,$B119)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A119,Aug2026!M3:M100,$B119)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A119,Sep2026!M3:M100,$B119)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A119,Oct2026!M3:M100,$B119)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A119,Nov2026!M3:M100,$B119)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A119,Dec2026!M3:M100,$B119)</f>
+        <v/>
+      </c>
+      <c r="D119" s="11" t="n"/>
+      <c r="G119" s="11" t="n"/>
+      <c r="J119" s="11" t="n"/>
+      <c r="M119" s="11" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="B120" s="11" t="inlineStr">
+        <is>
+          <t>Brochures</t>
+        </is>
+      </c>
+      <c r="C120" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A120,Jan2026!M3:M100,$B120)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A120,Feb2026!M3:M100,$B120)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A120,Mar2026!M3:M100,$B120)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A120,Apr2026!M3:M100,$B120)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A120,May2026!M3:M100,$B120)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A120,Jun2026!M3:M100,$B120)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A120,Jul2026!M3:M100,$B120)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A120,Aug2026!M3:M100,$B120)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A120,Sep2026!M3:M100,$B120)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A120,Oct2026!M3:M100,$B120)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A120,Nov2026!M3:M100,$B120)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A120,Dec2026!M3:M100,$B120)</f>
+        <v/>
+      </c>
+      <c r="D120" s="11" t="n"/>
+      <c r="G120" s="11" t="n"/>
+      <c r="J120" s="11" t="n"/>
+      <c r="M120" s="11" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="B121" s="11" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="C121" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A121,Jan2026!M3:M100,$B121)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A121,Feb2026!M3:M100,$B121)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A121,Mar2026!M3:M100,$B121)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A121,Apr2026!M3:M100,$B121)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A121,May2026!M3:M100,$B121)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A121,Jun2026!M3:M100,$B121)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A121,Jul2026!M3:M100,$B121)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A121,Aug2026!M3:M100,$B121)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A121,Sep2026!M3:M100,$B121)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A121,Oct2026!M3:M100,$B121)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A121,Nov2026!M3:M100,$B121)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A121,Dec2026!M3:M100,$B121)</f>
+        <v/>
+      </c>
+      <c r="D121" s="11" t="n"/>
+      <c r="G121" s="11" t="n"/>
+      <c r="J121" s="11" t="n"/>
+      <c r="M121" s="11" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="B122" s="11" t="inlineStr">
+        <is>
+          <t>Photography &amp; Drone</t>
+        </is>
+      </c>
+      <c r="C122" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A122,Jan2026!M3:M100,$B122)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A122,Feb2026!M3:M100,$B122)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A122,Mar2026!M3:M100,$B122)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A122,Apr2026!M3:M100,$B122)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A122,May2026!M3:M100,$B122)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A122,Jun2026!M3:M100,$B122)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A122,Jul2026!M3:M100,$B122)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A122,Aug2026!M3:M100,$B122)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A122,Sep2026!M3:M100,$B122)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A122,Oct2026!M3:M100,$B122)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A122,Nov2026!M3:M100,$B122)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A122,Dec2026!M3:M100,$B122)</f>
+        <v/>
+      </c>
+      <c r="D122" s="11" t="n"/>
+      <c r="G122" s="11" t="n"/>
+      <c r="J122" s="11" t="n"/>
+      <c r="M122" s="11" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="B123" s="11" t="inlineStr">
+        <is>
+          <t>Digital Marketing</t>
+        </is>
+      </c>
+      <c r="C123" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A123,Jan2026!M3:M100,$B123)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A123,Feb2026!M3:M100,$B123)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A123,Mar2026!M3:M100,$B123)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A123,Apr2026!M3:M100,$B123)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A123,May2026!M3:M100,$B123)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A123,Jun2026!M3:M100,$B123)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A123,Jul2026!M3:M100,$B123)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A123,Aug2026!M3:M100,$B123)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A123,Sep2026!M3:M100,$B123)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A123,Oct2026!M3:M100,$B123)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A123,Nov2026!M3:M100,$B123)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A123,Dec2026!M3:M100,$B123)</f>
+        <v/>
+      </c>
+      <c r="D123" s="11" t="n"/>
+      <c r="G123" s="11" t="n"/>
+      <c r="J123" s="11" t="n"/>
+      <c r="M123" s="11" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Miscellaneous</t>
+        </is>
+      </c>
+      <c r="B124" s="11" t="inlineStr">
+        <is>
+          <t>Travel Expenses</t>
+        </is>
+      </c>
+      <c r="C124" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A124,Jan2026!M3:M100,$B124)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A124,Feb2026!M3:M100,$B124)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A124,Mar2026!M3:M100,$B124)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A124,Apr2026!M3:M100,$B124)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A124,May2026!M3:M100,$B124)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A124,Jun2026!M3:M100,$B124)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A124,Jul2026!M3:M100,$B124)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A124,Aug2026!M3:M100,$B124)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A124,Sep2026!M3:M100,$B124)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A124,Oct2026!M3:M100,$B124)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A124,Nov2026!M3:M100,$B124)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A124,Dec2026!M3:M100,$B124)</f>
+        <v/>
+      </c>
+      <c r="D124" s="11" t="n"/>
+      <c r="G124" s="11" t="n"/>
+      <c r="J124" s="11" t="n"/>
+      <c r="M124" s="11" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Miscellaneous</t>
+        </is>
+      </c>
+      <c r="B125" s="11" t="inlineStr">
+        <is>
+          <t>Food &amp; Refreshments</t>
+        </is>
+      </c>
+      <c r="C125" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A125,Jan2026!M3:M100,$B125)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A125,Feb2026!M3:M100,$B125)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A125,Mar2026!M3:M100,$B125)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A125,Apr2026!M3:M100,$B125)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A125,May2026!M3:M100,$B125)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A125,Jun2026!M3:M100,$B125)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A125,Jul2026!M3:M100,$B125)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A125,Aug2026!M3:M100,$B125)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A125,Sep2026!M3:M100,$B125)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A125,Oct2026!M3:M100,$B125)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A125,Nov2026!M3:M100,$B125)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A125,Dec2026!M3:M100,$B125)</f>
+        <v/>
+      </c>
+      <c r="D125" s="11" t="n"/>
+      <c r="G125" s="11" t="n"/>
+      <c r="J125" s="11" t="n"/>
+      <c r="M125" s="11" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Miscellaneous</t>
+        </is>
+      </c>
+      <c r="B126" s="11" t="inlineStr">
+        <is>
+          <t>Government Fees</t>
+        </is>
+      </c>
+      <c r="C126" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A126,Jan2026!M3:M100,$B126)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A126,Feb2026!M3:M100,$B126)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A126,Mar2026!M3:M100,$B126)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A126,Apr2026!M3:M100,$B126)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A126,May2026!M3:M100,$B126)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A126,Jun2026!M3:M100,$B126)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A126,Jul2026!M3:M100,$B126)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A126,Aug2026!M3:M100,$B126)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A126,Sep2026!M3:M100,$B126)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A126,Oct2026!M3:M100,$B126)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A126,Nov2026!M3:M100,$B126)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A126,Dec2026!M3:M100,$B126)</f>
+        <v/>
+      </c>
+      <c r="D126" s="11" t="n"/>
+      <c r="G126" s="11" t="n"/>
+      <c r="J126" s="11" t="n"/>
+      <c r="M126" s="11" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Miscellaneous</t>
+        </is>
+      </c>
+      <c r="B127" s="11" t="inlineStr">
+        <is>
+          <t>Bank Charges</t>
+        </is>
+      </c>
+      <c r="C127" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A127,Jan2026!M3:M100,$B127)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A127,Feb2026!M3:M100,$B127)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A127,Mar2026!M3:M100,$B127)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A127,Apr2026!M3:M100,$B127)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A127,May2026!M3:M100,$B127)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A127,Jun2026!M3:M100,$B127)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A127,Jul2026!M3:M100,$B127)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A127,Aug2026!M3:M100,$B127)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A127,Sep2026!M3:M100,$B127)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A127,Oct2026!M3:M100,$B127)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A127,Nov2026!M3:M100,$B127)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A127,Dec2026!M3:M100,$B127)</f>
+        <v/>
+      </c>
+      <c r="D127" s="11" t="n"/>
+      <c r="G127" s="11" t="n"/>
+      <c r="J127" s="11" t="n"/>
+      <c r="M127" s="11" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Miscellaneous</t>
+        </is>
+      </c>
+      <c r="B128" s="11" t="inlineStr">
+        <is>
+          <t>Miscellaneous Expenses</t>
+        </is>
+      </c>
+      <c r="C128" s="11">
+        <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A128,Jan2026!M3:M100,$B128)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A128,Feb2026!M3:M100,$B128)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A128,Mar2026!M3:M100,$B128)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A128,Apr2026!M3:M100,$B128)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A128,May2026!M3:M100,$B128)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A128,Jun2026!M3:M100,$B128)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A128,Jul2026!M3:M100,$B128)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A128,Aug2026!M3:M100,$B128)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A128,Sep2026!M3:M100,$B128)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A128,Oct2026!M3:M100,$B128)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A128,Nov2026!M3:M100,$B128)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A128,Dec2026!M3:M100,$B128)</f>
+        <v/>
+      </c>
+      <c r="D128" s="11" t="n"/>
+      <c r="G128" s="11" t="n"/>
+      <c r="J128" s="11" t="n"/>
+      <c r="M128" s="11" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="5">
-    <dataValidation sqref="E3:E100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>='Categories'!$A$3:$A$6</formula1>
-    </dataValidation>
-    <dataValidation sqref="L3:L100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>='Categories'!$F$3:$F$12</formula1>
-    </dataValidation>
-    <dataValidation sqref="M3:M100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Sub-Category" error="Select a Main Category first, or pick a value that matches its sub-category list." type="list">
-      <formula1>INDIRECT("Cat_"&amp;SUBSTITUTE(SUBSTITUTE(L3," &amp; ","_")," ","_"))</formula1>
-    </dataValidation>
-    <dataValidation sqref="F3:F100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Bank,Cash"</formula1>
-    </dataValidation>
-    <dataValidation sqref="N3:N100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Bank,Cash"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -788,7 +2991,7 @@
         </is>
       </c>
       <c r="B103" s="7">
-        <f>'Sep2026'!B106</f>
+        <f>'Aug2026'!B106</f>
         <v/>
       </c>
     </row>
@@ -965,7 +3168,7 @@
         </is>
       </c>
       <c r="B103" s="7">
-        <f>'Oct2026'!B106</f>
+        <f>'Sep2026'!B106</f>
         <v/>
       </c>
     </row>
@@ -1142,7 +3345,7 @@
         </is>
       </c>
       <c r="B103" s="7">
-        <f>'Nov2026'!B106</f>
+        <f>'Oct2026'!B106</f>
         <v/>
       </c>
     </row>
@@ -1207,7 +3410,184 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q70"/>
+  <dimension ref="A1:O106"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Receipts</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SNO</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Receipts</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Payment Mode</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Main Category</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Sub-Category</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Payment Mode</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="1" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
+          <t>Opening Balance</t>
+        </is>
+      </c>
+      <c r="B103" s="7">
+        <f>'Nov2026'!B106</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
+          <t>Total Receipts</t>
+        </is>
+      </c>
+      <c r="B104" s="7">
+        <f>SUM(D3:D100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>Total Payments</t>
+        </is>
+      </c>
+      <c r="B105" s="7">
+        <f>SUM(K3:K100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="6" t="inlineStr">
+        <is>
+          <t>Net / Closing Balance</t>
+        </is>
+      </c>
+      <c r="B106" s="7">
+        <f>B103+B104-B105</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="5">
+    <dataValidation sqref="E3:E100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>='Categories'!$A$3:$A$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="L3:L100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>='Categories'!$F$3:$F$12</formula1>
+    </dataValidation>
+    <dataValidation sqref="M3:M100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Sub-Category" error="Select a Main Category first, or pick a value that matches its sub-category list." type="list">
+      <formula1>INDIRECT("Cat_"&amp;SUBSTITUTE(SUBSTITUTE(L3," &amp; ","_")," ","_"))</formula1>
+    </dataValidation>
+    <dataValidation sqref="F3:F100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Bank,Cash"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N3:N100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Bank,Cash"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2668,9 +5048,8 @@
           <t>Opening Balance</t>
         </is>
       </c>
-      <c r="B103" s="7">
-        <f>'Jan2026'!B106</f>
-        <v/>
+      <c r="B103" s="7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="104">
@@ -2846,7 +5225,7 @@
         </is>
       </c>
       <c r="B103" s="7">
-        <f>'Feb2026'!B106</f>
+        <f>'Jan2026'!B106</f>
         <v/>
       </c>
     </row>
@@ -3023,7 +5402,7 @@
         </is>
       </c>
       <c r="B103" s="7">
-        <f>'Mar2026'!B106</f>
+        <f>'Feb2026'!B106</f>
         <v/>
       </c>
     </row>
@@ -3200,7 +5579,7 @@
         </is>
       </c>
       <c r="B103" s="7">
-        <f>'Apr2026'!B106</f>
+        <f>'Mar2026'!B106</f>
         <v/>
       </c>
     </row>
@@ -3377,7 +5756,7 @@
         </is>
       </c>
       <c r="B103" s="7">
-        <f>'May2026'!B106</f>
+        <f>'Apr2026'!B106</f>
         <v/>
       </c>
     </row>
@@ -3554,7 +5933,7 @@
         </is>
       </c>
       <c r="B103" s="7">
-        <f>'Jun2026'!B106</f>
+        <f>'May2026'!B106</f>
         <v/>
       </c>
     </row>
@@ -3731,7 +6110,7 @@
         </is>
       </c>
       <c r="B103" s="7">
-        <f>'Jul2026'!B106</f>
+        <f>'Jun2026'!B106</f>
         <v/>
       </c>
     </row>
@@ -3908,7 +6287,7 @@
         </is>
       </c>
       <c r="B103" s="7">
-        <f>'Aug2026'!B106</f>
+        <f>'Jul2026'!B106</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Dashboard styling: apply green/red palette to receipts/payments elements, precise number-format ranges
- Apply palette colors to KPI labels: green (2E7D32) for YTD Receipts, red (C62828) for YTD Payments, slate (37474F) for neutral elements
- Color Monthly Trend table headers: green for Receipts, red for Payments, slate for Month and Closing Balance
- Color category table headers: green for Income Category (receipts-side), red for Main Category (expense-side) and Sub-Category Detail
- Keep Bank vs Cash header slate (neutral, mixes receipts and payments)
- Replace imprecise number-format loop with precise column/row ranges for each table
- All 7 tests pass; Dashboard styling matches design spec palette requirements
</commit_message>
<xml_diff>
--- a/expense_tracker_2026.xlsx
+++ b/expense_tracker_2026.xlsx
@@ -129,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -150,6 +150,12 @@
     </xf>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -981,12 +987,12 @@
           <t>Current Cash Balance</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>YTD Total Receipts</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>YTD Total Payments</t>
         </is>
@@ -1021,12 +1027,12 @@
           <t>Month</t>
         </is>
       </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Receipts</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>Payments</t>
         </is>
@@ -1036,22 +1042,22 @@
           <t>Closing Balance</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="F44" s="3" t="inlineStr">
         <is>
           <t>Main Category</t>
         </is>
       </c>
-      <c r="G44" s="4" t="inlineStr">
+      <c r="G44" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="I44" s="4" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>Income Category</t>
         </is>
       </c>
-      <c r="J44" s="4" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
@@ -1195,7 +1201,6 @@
         <f>SUMIFS(Jan2026!D3:D100,Jan2026!E3:E100,$I47)+SUMIFS(Feb2026!D3:D100,Feb2026!E3:E100,$I47)+SUMIFS(Mar2026!D3:D100,Mar2026!E3:E100,$I47)+SUMIFS(Apr2026!D3:D100,Apr2026!E3:E100,$I47)+SUMIFS(May2026!D3:D100,May2026!E3:E100,$I47)+SUMIFS(Jun2026!D3:D100,Jun2026!E3:E100,$I47)+SUMIFS(Jul2026!D3:D100,Jul2026!E3:E100,$I47)+SUMIFS(Aug2026!D3:D100,Aug2026!E3:E100,$I47)+SUMIFS(Sep2026!D3:D100,Sep2026!E3:E100,$I47)+SUMIFS(Oct2026!D3:D100,Oct2026!E3:E100,$I47)+SUMIFS(Nov2026!D3:D100,Nov2026!E3:E100,$I47)+SUMIFS(Dec2026!D3:D100,Dec2026!E3:E100,$I47)</f>
         <v/>
       </c>
-      <c r="M47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1233,7 +1238,6 @@
         <f>SUMIFS(Jan2026!D3:D100,Jan2026!E3:E100,$I48)+SUMIFS(Feb2026!D3:D100,Feb2026!E3:E100,$I48)+SUMIFS(Mar2026!D3:D100,Mar2026!E3:E100,$I48)+SUMIFS(Apr2026!D3:D100,Apr2026!E3:E100,$I48)+SUMIFS(May2026!D3:D100,May2026!E3:E100,$I48)+SUMIFS(Jun2026!D3:D100,Jun2026!E3:E100,$I48)+SUMIFS(Jul2026!D3:D100,Jul2026!E3:E100,$I48)+SUMIFS(Aug2026!D3:D100,Aug2026!E3:E100,$I48)+SUMIFS(Sep2026!D3:D100,Sep2026!E3:E100,$I48)+SUMIFS(Oct2026!D3:D100,Oct2026!E3:E100,$I48)+SUMIFS(Nov2026!D3:D100,Nov2026!E3:E100,$I48)+SUMIFS(Dec2026!D3:D100,Dec2026!E3:E100,$I48)</f>
         <v/>
       </c>
-      <c r="M48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1262,8 +1266,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F49)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F49)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F49)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F49)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F49)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F49)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F49)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F49)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F49)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F49)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F49)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F49)</f>
         <v/>
       </c>
-      <c r="J49" s="11" t="n"/>
-      <c r="M49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1292,8 +1294,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F50)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F50)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F50)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F50)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F50)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F50)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F50)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F50)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F50)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F50)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F50)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F50)</f>
         <v/>
       </c>
-      <c r="J50" s="11" t="n"/>
-      <c r="M50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1322,8 +1322,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F51)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F51)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F51)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F51)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F51)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F51)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F51)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F51)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F51)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F51)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F51)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F51)</f>
         <v/>
       </c>
-      <c r="J51" s="11" t="n"/>
-      <c r="M51" s="11" t="n"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1352,8 +1350,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F52)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F52)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F52)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F52)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F52)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F52)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F52)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F52)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F52)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F52)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F52)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F52)</f>
         <v/>
       </c>
-      <c r="J52" s="11" t="n"/>
-      <c r="M52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1382,8 +1378,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F53)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F53)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F53)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F53)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F53)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F53)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F53)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F53)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F53)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F53)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F53)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F53)</f>
         <v/>
       </c>
-      <c r="J53" s="11" t="n"/>
-      <c r="M53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1412,8 +1406,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$F54)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$F54)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$F54)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$F54)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$F54)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$F54)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$F54)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$F54)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$F54)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$F54)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$F54)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$F54)</f>
         <v/>
       </c>
-      <c r="J54" s="11" t="n"/>
-      <c r="M54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1433,9 +1425,6 @@
         <f>'Nov2026'!B106</f>
         <v/>
       </c>
-      <c r="G55" s="11" t="n"/>
-      <c r="J55" s="11" t="n"/>
-      <c r="M55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1455,54 +1444,23 @@
         <f>'Dec2026'!B106</f>
         <v/>
       </c>
-      <c r="G56" s="11" t="n"/>
-      <c r="J56" s="11" t="n"/>
-      <c r="M56" s="11" t="n"/>
-    </row>
-    <row r="57">
-      <c r="B57" s="11" t="n"/>
-      <c r="C57" s="11" t="n"/>
-      <c r="D57" s="11" t="n"/>
-      <c r="G57" s="11" t="n"/>
-      <c r="J57" s="11" t="n"/>
-      <c r="M57" s="11" t="n"/>
-    </row>
-    <row r="58">
-      <c r="B58" s="11" t="n"/>
-      <c r="C58" s="11" t="n"/>
-      <c r="D58" s="11" t="n"/>
-      <c r="G58" s="11" t="n"/>
-      <c r="J58" s="11" t="n"/>
-      <c r="M58" s="11" t="n"/>
-    </row>
-    <row r="59">
-      <c r="B59" s="11" t="n"/>
-      <c r="C59" s="11" t="n"/>
-      <c r="D59" s="11" t="n"/>
-      <c r="G59" s="11" t="n"/>
-      <c r="J59" s="11" t="n"/>
-      <c r="M59" s="11" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>Main Category</t>
         </is>
       </c>
-      <c r="B60" s="11" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>Sub-Category</t>
         </is>
       </c>
-      <c r="C60" s="11" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D60" s="11" t="n"/>
-      <c r="G60" s="11" t="n"/>
-      <c r="J60" s="11" t="n"/>
-      <c r="M60" s="11" t="n"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1510,7 +1468,7 @@
           <t>Land &amp; Legal</t>
         </is>
       </c>
-      <c r="B61" s="11" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>Land Purchase</t>
         </is>
@@ -1519,10 +1477,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A61,Jan2026!M3:M100,$B61)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A61,Feb2026!M3:M100,$B61)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A61,Mar2026!M3:M100,$B61)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A61,Apr2026!M3:M100,$B61)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A61,May2026!M3:M100,$B61)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A61,Jun2026!M3:M100,$B61)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A61,Jul2026!M3:M100,$B61)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A61,Aug2026!M3:M100,$B61)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A61,Sep2026!M3:M100,$B61)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A61,Oct2026!M3:M100,$B61)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A61,Nov2026!M3:M100,$B61)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A61,Dec2026!M3:M100,$B61)</f>
         <v/>
       </c>
-      <c r="D61" s="11" t="n"/>
-      <c r="G61" s="11" t="n"/>
-      <c r="J61" s="11" t="n"/>
-      <c r="M61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1530,7 +1484,7 @@
           <t>Land &amp; Legal</t>
         </is>
       </c>
-      <c r="B62" s="11" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>Advance Payments</t>
         </is>
@@ -1539,10 +1493,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A62,Jan2026!M3:M100,$B62)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A62,Feb2026!M3:M100,$B62)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A62,Mar2026!M3:M100,$B62)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A62,Apr2026!M3:M100,$B62)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A62,May2026!M3:M100,$B62)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A62,Jun2026!M3:M100,$B62)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A62,Jul2026!M3:M100,$B62)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A62,Aug2026!M3:M100,$B62)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A62,Sep2026!M3:M100,$B62)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A62,Oct2026!M3:M100,$B62)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A62,Nov2026!M3:M100,$B62)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A62,Dec2026!M3:M100,$B62)</f>
         <v/>
       </c>
-      <c r="D62" s="11" t="n"/>
-      <c r="G62" s="11" t="n"/>
-      <c r="J62" s="11" t="n"/>
-      <c r="M62" s="11" t="n"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1550,7 +1500,7 @@
           <t>Land &amp; Legal</t>
         </is>
       </c>
-      <c r="B63" s="11" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>Registration Charges</t>
         </is>
@@ -1559,10 +1509,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A63,Jan2026!M3:M100,$B63)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A63,Feb2026!M3:M100,$B63)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A63,Mar2026!M3:M100,$B63)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A63,Apr2026!M3:M100,$B63)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A63,May2026!M3:M100,$B63)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A63,Jun2026!M3:M100,$B63)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A63,Jul2026!M3:M100,$B63)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A63,Aug2026!M3:M100,$B63)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A63,Sep2026!M3:M100,$B63)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A63,Oct2026!M3:M100,$B63)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A63,Nov2026!M3:M100,$B63)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A63,Dec2026!M3:M100,$B63)</f>
         <v/>
       </c>
-      <c r="D63" s="11" t="n"/>
-      <c r="G63" s="11" t="n"/>
-      <c r="J63" s="11" t="n"/>
-      <c r="M63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1570,7 +1516,7 @@
           <t>Land &amp; Legal</t>
         </is>
       </c>
-      <c r="B64" s="11" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>Stamp Duty</t>
         </is>
@@ -1579,10 +1525,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A64,Jan2026!M3:M100,$B64)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A64,Feb2026!M3:M100,$B64)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A64,Mar2026!M3:M100,$B64)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A64,Apr2026!M3:M100,$B64)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A64,May2026!M3:M100,$B64)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A64,Jun2026!M3:M100,$B64)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A64,Jul2026!M3:M100,$B64)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A64,Aug2026!M3:M100,$B64)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A64,Sep2026!M3:M100,$B64)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A64,Oct2026!M3:M100,$B64)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A64,Nov2026!M3:M100,$B64)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A64,Dec2026!M3:M100,$B64)</f>
         <v/>
       </c>
-      <c r="D64" s="11" t="n"/>
-      <c r="G64" s="11" t="n"/>
-      <c r="J64" s="11" t="n"/>
-      <c r="M64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1590,7 +1532,7 @@
           <t>Land &amp; Legal</t>
         </is>
       </c>
-      <c r="B65" s="11" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>Legal Fees</t>
         </is>
@@ -1599,10 +1541,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A65,Jan2026!M3:M100,$B65)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A65,Feb2026!M3:M100,$B65)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A65,Mar2026!M3:M100,$B65)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A65,Apr2026!M3:M100,$B65)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A65,May2026!M3:M100,$B65)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A65,Jun2026!M3:M100,$B65)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A65,Jul2026!M3:M100,$B65)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A65,Aug2026!M3:M100,$B65)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A65,Sep2026!M3:M100,$B65)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A65,Oct2026!M3:M100,$B65)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A65,Nov2026!M3:M100,$B65)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A65,Dec2026!M3:M100,$B65)</f>
         <v/>
       </c>
-      <c r="D65" s="11" t="n"/>
-      <c r="G65" s="11" t="n"/>
-      <c r="J65" s="11" t="n"/>
-      <c r="M65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1610,7 +1548,7 @@
           <t>Land &amp; Legal</t>
         </is>
       </c>
-      <c r="B66" s="11" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>Survey Charges</t>
         </is>
@@ -1619,10 +1557,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A66,Jan2026!M3:M100,$B66)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A66,Feb2026!M3:M100,$B66)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A66,Mar2026!M3:M100,$B66)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A66,Apr2026!M3:M100,$B66)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A66,May2026!M3:M100,$B66)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A66,Jun2026!M3:M100,$B66)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A66,Jul2026!M3:M100,$B66)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A66,Aug2026!M3:M100,$B66)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A66,Sep2026!M3:M100,$B66)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A66,Oct2026!M3:M100,$B66)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A66,Nov2026!M3:M100,$B66)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A66,Dec2026!M3:M100,$B66)</f>
         <v/>
       </c>
-      <c r="D66" s="11" t="n"/>
-      <c r="G66" s="11" t="n"/>
-      <c r="J66" s="11" t="n"/>
-      <c r="M66" s="11" t="n"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1630,7 +1564,7 @@
           <t>Land &amp; Legal</t>
         </is>
       </c>
-      <c r="B67" s="11" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
@@ -1639,10 +1573,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A67,Jan2026!M3:M100,$B67)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A67,Feb2026!M3:M100,$B67)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A67,Mar2026!M3:M100,$B67)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A67,Apr2026!M3:M100,$B67)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A67,May2026!M3:M100,$B67)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A67,Jun2026!M3:M100,$B67)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A67,Jul2026!M3:M100,$B67)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A67,Aug2026!M3:M100,$B67)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A67,Sep2026!M3:M100,$B67)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A67,Oct2026!M3:M100,$B67)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A67,Nov2026!M3:M100,$B67)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A67,Dec2026!M3:M100,$B67)</f>
         <v/>
       </c>
-      <c r="D67" s="11" t="n"/>
-      <c r="G67" s="11" t="n"/>
-      <c r="J67" s="11" t="n"/>
-      <c r="M67" s="11" t="n"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1650,7 +1580,7 @@
           <t>Site Development</t>
         </is>
       </c>
-      <c r="B68" s="11" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>Land Clearing</t>
         </is>
@@ -1659,10 +1589,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A68,Jan2026!M3:M100,$B68)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A68,Feb2026!M3:M100,$B68)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A68,Mar2026!M3:M100,$B68)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A68,Apr2026!M3:M100,$B68)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A68,May2026!M3:M100,$B68)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A68,Jun2026!M3:M100,$B68)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A68,Jul2026!M3:M100,$B68)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A68,Aug2026!M3:M100,$B68)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A68,Sep2026!M3:M100,$B68)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A68,Oct2026!M3:M100,$B68)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A68,Nov2026!M3:M100,$B68)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A68,Dec2026!M3:M100,$B68)</f>
         <v/>
       </c>
-      <c r="D68" s="11" t="n"/>
-      <c r="G68" s="11" t="n"/>
-      <c r="J68" s="11" t="n"/>
-      <c r="M68" s="11" t="n"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1670,7 +1596,7 @@
           <t>Site Development</t>
         </is>
       </c>
-      <c r="B69" s="11" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t>Earthwork &amp; Levelling</t>
         </is>
@@ -1679,10 +1605,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A69,Jan2026!M3:M100,$B69)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A69,Feb2026!M3:M100,$B69)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A69,Mar2026!M3:M100,$B69)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A69,Apr2026!M3:M100,$B69)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A69,May2026!M3:M100,$B69)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A69,Jun2026!M3:M100,$B69)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A69,Jul2026!M3:M100,$B69)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A69,Aug2026!M3:M100,$B69)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A69,Sep2026!M3:M100,$B69)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A69,Oct2026!M3:M100,$B69)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A69,Nov2026!M3:M100,$B69)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A69,Dec2026!M3:M100,$B69)</f>
         <v/>
       </c>
-      <c r="D69" s="11" t="n"/>
-      <c r="G69" s="11" t="n"/>
-      <c r="J69" s="11" t="n"/>
-      <c r="M69" s="11" t="n"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1690,7 +1612,7 @@
           <t>Site Development</t>
         </is>
       </c>
-      <c r="B70" s="11" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t>Road Formation</t>
         </is>
@@ -1699,10 +1621,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A70,Jan2026!M3:M100,$B70)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A70,Feb2026!M3:M100,$B70)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A70,Mar2026!M3:M100,$B70)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A70,Apr2026!M3:M100,$B70)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A70,May2026!M3:M100,$B70)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A70,Jun2026!M3:M100,$B70)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A70,Jul2026!M3:M100,$B70)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A70,Aug2026!M3:M100,$B70)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A70,Sep2026!M3:M100,$B70)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A70,Oct2026!M3:M100,$B70)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A70,Nov2026!M3:M100,$B70)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A70,Dec2026!M3:M100,$B70)</f>
         <v/>
       </c>
-      <c r="D70" s="11" t="n"/>
-      <c r="G70" s="11" t="n"/>
-      <c r="J70" s="11" t="n"/>
-      <c r="M70" s="11" t="n"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1710,7 +1628,7 @@
           <t>Site Development</t>
         </is>
       </c>
-      <c r="B71" s="11" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t>Blacktop Roads</t>
         </is>
@@ -1719,10 +1637,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A71,Jan2026!M3:M100,$B71)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A71,Feb2026!M3:M100,$B71)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A71,Mar2026!M3:M100,$B71)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A71,Apr2026!M3:M100,$B71)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A71,May2026!M3:M100,$B71)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A71,Jun2026!M3:M100,$B71)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A71,Jul2026!M3:M100,$B71)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A71,Aug2026!M3:M100,$B71)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A71,Sep2026!M3:M100,$B71)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A71,Oct2026!M3:M100,$B71)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A71,Nov2026!M3:M100,$B71)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A71,Dec2026!M3:M100,$B71)</f>
         <v/>
       </c>
-      <c r="D71" s="11" t="n"/>
-      <c r="G71" s="11" t="n"/>
-      <c r="J71" s="11" t="n"/>
-      <c r="M71" s="11" t="n"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1730,7 +1644,7 @@
           <t>Site Development</t>
         </is>
       </c>
-      <c r="B72" s="11" t="inlineStr">
+      <c r="B72" t="inlineStr">
         <is>
           <t>Interlocking Pavers</t>
         </is>
@@ -1739,10 +1653,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A72,Jan2026!M3:M100,$B72)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A72,Feb2026!M3:M100,$B72)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A72,Mar2026!M3:M100,$B72)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A72,Apr2026!M3:M100,$B72)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A72,May2026!M3:M100,$B72)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A72,Jun2026!M3:M100,$B72)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A72,Jul2026!M3:M100,$B72)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A72,Aug2026!M3:M100,$B72)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A72,Sep2026!M3:M100,$B72)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A72,Oct2026!M3:M100,$B72)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A72,Nov2026!M3:M100,$B72)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A72,Dec2026!M3:M100,$B72)</f>
         <v/>
       </c>
-      <c r="D72" s="11" t="n"/>
-      <c r="G72" s="11" t="n"/>
-      <c r="J72" s="11" t="n"/>
-      <c r="M72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1750,7 +1660,7 @@
           <t>Site Development</t>
         </is>
       </c>
-      <c r="B73" s="11" t="inlineStr">
+      <c r="B73" t="inlineStr">
         <is>
           <t>Compound Wall</t>
         </is>
@@ -1759,10 +1669,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A73,Jan2026!M3:M100,$B73)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A73,Feb2026!M3:M100,$B73)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A73,Mar2026!M3:M100,$B73)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A73,Apr2026!M3:M100,$B73)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A73,May2026!M3:M100,$B73)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A73,Jun2026!M3:M100,$B73)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A73,Jul2026!M3:M100,$B73)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A73,Aug2026!M3:M100,$B73)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A73,Sep2026!M3:M100,$B73)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A73,Oct2026!M3:M100,$B73)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A73,Nov2026!M3:M100,$B73)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A73,Dec2026!M3:M100,$B73)</f>
         <v/>
       </c>
-      <c r="D73" s="11" t="n"/>
-      <c r="G73" s="11" t="n"/>
-      <c r="J73" s="11" t="n"/>
-      <c r="M73" s="11" t="n"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1770,7 +1676,7 @@
           <t>Site Development</t>
         </is>
       </c>
-      <c r="B74" s="11" t="inlineStr">
+      <c r="B74" t="inlineStr">
         <is>
           <t>Entrance Gate</t>
         </is>
@@ -1779,10 +1685,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A74,Jan2026!M3:M100,$B74)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A74,Feb2026!M3:M100,$B74)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A74,Mar2026!M3:M100,$B74)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A74,Apr2026!M3:M100,$B74)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A74,May2026!M3:M100,$B74)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A74,Jun2026!M3:M100,$B74)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A74,Jul2026!M3:M100,$B74)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A74,Aug2026!M3:M100,$B74)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A74,Sep2026!M3:M100,$B74)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A74,Oct2026!M3:M100,$B74)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A74,Nov2026!M3:M100,$B74)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A74,Dec2026!M3:M100,$B74)</f>
         <v/>
       </c>
-      <c r="D74" s="11" t="n"/>
-      <c r="G74" s="11" t="n"/>
-      <c r="J74" s="11" t="n"/>
-      <c r="M74" s="11" t="n"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1790,7 +1692,7 @@
           <t>Site Development</t>
         </is>
       </c>
-      <c r="B75" s="11" t="inlineStr">
+      <c r="B75" t="inlineStr">
         <is>
           <t>Drainage</t>
         </is>
@@ -1799,10 +1701,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A75,Jan2026!M3:M100,$B75)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A75,Feb2026!M3:M100,$B75)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A75,Mar2026!M3:M100,$B75)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A75,Apr2026!M3:M100,$B75)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A75,May2026!M3:M100,$B75)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A75,Jun2026!M3:M100,$B75)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A75,Jul2026!M3:M100,$B75)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A75,Aug2026!M3:M100,$B75)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A75,Sep2026!M3:M100,$B75)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A75,Oct2026!M3:M100,$B75)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A75,Nov2026!M3:M100,$B75)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A75,Dec2026!M3:M100,$B75)</f>
         <v/>
       </c>
-      <c r="D75" s="11" t="n"/>
-      <c r="G75" s="11" t="n"/>
-      <c r="J75" s="11" t="n"/>
-      <c r="M75" s="11" t="n"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1810,7 +1708,7 @@
           <t>Site Development</t>
         </is>
       </c>
-      <c r="B76" s="11" t="inlineStr">
+      <c r="B76" t="inlineStr">
         <is>
           <t>Culverts</t>
         </is>
@@ -1819,10 +1717,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A76,Jan2026!M3:M100,$B76)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A76,Feb2026!M3:M100,$B76)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A76,Mar2026!M3:M100,$B76)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A76,Apr2026!M3:M100,$B76)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A76,May2026!M3:M100,$B76)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A76,Jun2026!M3:M100,$B76)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A76,Jul2026!M3:M100,$B76)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A76,Aug2026!M3:M100,$B76)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A76,Sep2026!M3:M100,$B76)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A76,Oct2026!M3:M100,$B76)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A76,Nov2026!M3:M100,$B76)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A76,Dec2026!M3:M100,$B76)</f>
         <v/>
       </c>
-      <c r="D76" s="11" t="n"/>
-      <c r="G76" s="11" t="n"/>
-      <c r="J76" s="11" t="n"/>
-      <c r="M76" s="11" t="n"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1830,7 +1724,7 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="B77" s="11" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t>Borewell</t>
         </is>
@@ -1839,10 +1733,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A77,Jan2026!M3:M100,$B77)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A77,Feb2026!M3:M100,$B77)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A77,Mar2026!M3:M100,$B77)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A77,Apr2026!M3:M100,$B77)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A77,May2026!M3:M100,$B77)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A77,Jun2026!M3:M100,$B77)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A77,Jul2026!M3:M100,$B77)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A77,Aug2026!M3:M100,$B77)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A77,Sep2026!M3:M100,$B77)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A77,Oct2026!M3:M100,$B77)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A77,Nov2026!M3:M100,$B77)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A77,Dec2026!M3:M100,$B77)</f>
         <v/>
       </c>
-      <c r="D77" s="11" t="n"/>
-      <c r="G77" s="11" t="n"/>
-      <c r="J77" s="11" t="n"/>
-      <c r="M77" s="11" t="n"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1850,7 +1740,7 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="B78" s="11" t="inlineStr">
+      <c r="B78" t="inlineStr">
         <is>
           <t>Water Pipelines</t>
         </is>
@@ -1859,10 +1749,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A78,Jan2026!M3:M100,$B78)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A78,Feb2026!M3:M100,$B78)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A78,Mar2026!M3:M100,$B78)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A78,Apr2026!M3:M100,$B78)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A78,May2026!M3:M100,$B78)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A78,Jun2026!M3:M100,$B78)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A78,Jul2026!M3:M100,$B78)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A78,Aug2026!M3:M100,$B78)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A78,Sep2026!M3:M100,$B78)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A78,Oct2026!M3:M100,$B78)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A78,Nov2026!M3:M100,$B78)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A78,Dec2026!M3:M100,$B78)</f>
         <v/>
       </c>
-      <c r="D78" s="11" t="n"/>
-      <c r="G78" s="11" t="n"/>
-      <c r="J78" s="11" t="n"/>
-      <c r="M78" s="11" t="n"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1870,7 +1756,7 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="B79" s="11" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>Water Tank</t>
         </is>
@@ -1879,10 +1765,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A79,Jan2026!M3:M100,$B79)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A79,Feb2026!M3:M100,$B79)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A79,Mar2026!M3:M100,$B79)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A79,Apr2026!M3:M100,$B79)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A79,May2026!M3:M100,$B79)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A79,Jun2026!M3:M100,$B79)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A79,Jul2026!M3:M100,$B79)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A79,Aug2026!M3:M100,$B79)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A79,Sep2026!M3:M100,$B79)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A79,Oct2026!M3:M100,$B79)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A79,Nov2026!M3:M100,$B79)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A79,Dec2026!M3:M100,$B79)</f>
         <v/>
       </c>
-      <c r="D79" s="11" t="n"/>
-      <c r="G79" s="11" t="n"/>
-      <c r="J79" s="11" t="n"/>
-      <c r="M79" s="11" t="n"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1890,7 +1772,7 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="B80" s="11" t="inlineStr">
+      <c r="B80" t="inlineStr">
         <is>
           <t>Electricity Connection</t>
         </is>
@@ -1899,10 +1781,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A80,Jan2026!M3:M100,$B80)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A80,Feb2026!M3:M100,$B80)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A80,Mar2026!M3:M100,$B80)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A80,Apr2026!M3:M100,$B80)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A80,May2026!M3:M100,$B80)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A80,Jun2026!M3:M100,$B80)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A80,Jul2026!M3:M100,$B80)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A80,Aug2026!M3:M100,$B80)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A80,Sep2026!M3:M100,$B80)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A80,Oct2026!M3:M100,$B80)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A80,Nov2026!M3:M100,$B80)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A80,Dec2026!M3:M100,$B80)</f>
         <v/>
       </c>
-      <c r="D80" s="11" t="n"/>
-      <c r="G80" s="11" t="n"/>
-      <c r="J80" s="11" t="n"/>
-      <c r="M80" s="11" t="n"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1910,7 +1788,7 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="B81" s="11" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>Transformer</t>
         </is>
@@ -1919,10 +1797,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A81,Jan2026!M3:M100,$B81)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A81,Feb2026!M3:M100,$B81)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A81,Mar2026!M3:M100,$B81)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A81,Apr2026!M3:M100,$B81)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A81,May2026!M3:M100,$B81)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A81,Jun2026!M3:M100,$B81)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A81,Jul2026!M3:M100,$B81)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A81,Aug2026!M3:M100,$B81)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A81,Sep2026!M3:M100,$B81)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A81,Oct2026!M3:M100,$B81)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A81,Nov2026!M3:M100,$B81)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A81,Dec2026!M3:M100,$B81)</f>
         <v/>
       </c>
-      <c r="D81" s="11" t="n"/>
-      <c r="G81" s="11" t="n"/>
-      <c r="J81" s="11" t="n"/>
-      <c r="M81" s="11" t="n"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1930,7 +1804,7 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="B82" s="11" t="inlineStr">
+      <c r="B82" t="inlineStr">
         <is>
           <t>Street Lights</t>
         </is>
@@ -1939,10 +1813,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A82,Jan2026!M3:M100,$B82)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A82,Feb2026!M3:M100,$B82)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A82,Mar2026!M3:M100,$B82)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A82,Apr2026!M3:M100,$B82)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A82,May2026!M3:M100,$B82)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A82,Jun2026!M3:M100,$B82)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A82,Jul2026!M3:M100,$B82)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A82,Aug2026!M3:M100,$B82)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A82,Sep2026!M3:M100,$B82)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A82,Oct2026!M3:M100,$B82)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A82,Nov2026!M3:M100,$B82)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A82,Dec2026!M3:M100,$B82)</f>
         <v/>
       </c>
-      <c r="D82" s="11" t="n"/>
-      <c r="G82" s="11" t="n"/>
-      <c r="J82" s="11" t="n"/>
-      <c r="M82" s="11" t="n"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1950,7 +1820,7 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="B83" s="11" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>Generator</t>
         </is>
@@ -1959,10 +1829,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A83,Jan2026!M3:M100,$B83)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A83,Feb2026!M3:M100,$B83)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A83,Mar2026!M3:M100,$B83)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A83,Apr2026!M3:M100,$B83)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A83,May2026!M3:M100,$B83)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A83,Jun2026!M3:M100,$B83)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A83,Jul2026!M3:M100,$B83)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A83,Aug2026!M3:M100,$B83)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A83,Sep2026!M3:M100,$B83)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A83,Oct2026!M3:M100,$B83)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A83,Nov2026!M3:M100,$B83)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A83,Dec2026!M3:M100,$B83)</f>
         <v/>
       </c>
-      <c r="D83" s="11" t="n"/>
-      <c r="G83" s="11" t="n"/>
-      <c r="J83" s="11" t="n"/>
-      <c r="M83" s="11" t="n"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1970,7 +1836,7 @@
           <t>Landscaping</t>
         </is>
       </c>
-      <c r="B84" s="11" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>Plantation</t>
         </is>
@@ -1979,10 +1845,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A84,Jan2026!M3:M100,$B84)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A84,Feb2026!M3:M100,$B84)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A84,Mar2026!M3:M100,$B84)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A84,Apr2026!M3:M100,$B84)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A84,May2026!M3:M100,$B84)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A84,Jun2026!M3:M100,$B84)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A84,Jul2026!M3:M100,$B84)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A84,Aug2026!M3:M100,$B84)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A84,Sep2026!M3:M100,$B84)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A84,Oct2026!M3:M100,$B84)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A84,Nov2026!M3:M100,$B84)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A84,Dec2026!M3:M100,$B84)</f>
         <v/>
       </c>
-      <c r="D84" s="11" t="n"/>
-      <c r="G84" s="11" t="n"/>
-      <c r="J84" s="11" t="n"/>
-      <c r="M84" s="11" t="n"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1990,7 +1852,7 @@
           <t>Landscaping</t>
         </is>
       </c>
-      <c r="B85" s="11" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>Miyawaki Forest</t>
         </is>
@@ -1999,10 +1861,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A85,Jan2026!M3:M100,$B85)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A85,Feb2026!M3:M100,$B85)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A85,Mar2026!M3:M100,$B85)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A85,Apr2026!M3:M100,$B85)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A85,May2026!M3:M100,$B85)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A85,Jun2026!M3:M100,$B85)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A85,Jul2026!M3:M100,$B85)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A85,Aug2026!M3:M100,$B85)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A85,Sep2026!M3:M100,$B85)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A85,Oct2026!M3:M100,$B85)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A85,Nov2026!M3:M100,$B85)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A85,Dec2026!M3:M100,$B85)</f>
         <v/>
       </c>
-      <c r="D85" s="11" t="n"/>
-      <c r="G85" s="11" t="n"/>
-      <c r="J85" s="11" t="n"/>
-      <c r="M85" s="11" t="n"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2010,7 +1868,7 @@
           <t>Landscaping</t>
         </is>
       </c>
-      <c r="B86" s="11" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>Lawn Development</t>
         </is>
@@ -2019,10 +1877,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A86,Jan2026!M3:M100,$B86)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A86,Feb2026!M3:M100,$B86)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A86,Mar2026!M3:M100,$B86)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A86,Apr2026!M3:M100,$B86)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A86,May2026!M3:M100,$B86)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A86,Jun2026!M3:M100,$B86)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A86,Jul2026!M3:M100,$B86)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A86,Aug2026!M3:M100,$B86)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A86,Sep2026!M3:M100,$B86)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A86,Oct2026!M3:M100,$B86)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A86,Nov2026!M3:M100,$B86)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A86,Dec2026!M3:M100,$B86)</f>
         <v/>
       </c>
-      <c r="D86" s="11" t="n"/>
-      <c r="G86" s="11" t="n"/>
-      <c r="J86" s="11" t="n"/>
-      <c r="M86" s="11" t="n"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2030,7 +1884,7 @@
           <t>Landscaping</t>
         </is>
       </c>
-      <c r="B87" s="11" t="inlineStr">
+      <c r="B87" t="inlineStr">
         <is>
           <t>Irrigation/Drip System</t>
         </is>
@@ -2039,10 +1893,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A87,Jan2026!M3:M100,$B87)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A87,Feb2026!M3:M100,$B87)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A87,Mar2026!M3:M100,$B87)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A87,Apr2026!M3:M100,$B87)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A87,May2026!M3:M100,$B87)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A87,Jun2026!M3:M100,$B87)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A87,Jul2026!M3:M100,$B87)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A87,Aug2026!M3:M100,$B87)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A87,Sep2026!M3:M100,$B87)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A87,Oct2026!M3:M100,$B87)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A87,Nov2026!M3:M100,$B87)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A87,Dec2026!M3:M100,$B87)</f>
         <v/>
       </c>
-      <c r="D87" s="11" t="n"/>
-      <c r="G87" s="11" t="n"/>
-      <c r="J87" s="11" t="n"/>
-      <c r="M87" s="11" t="n"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2050,7 +1900,7 @@
           <t>Landscaping</t>
         </is>
       </c>
-      <c r="B88" s="11" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t>Garden Maintenance</t>
         </is>
@@ -2059,10 +1909,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A88,Jan2026!M3:M100,$B88)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A88,Feb2026!M3:M100,$B88)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A88,Mar2026!M3:M100,$B88)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A88,Apr2026!M3:M100,$B88)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A88,May2026!M3:M100,$B88)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A88,Jun2026!M3:M100,$B88)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A88,Jul2026!M3:M100,$B88)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A88,Aug2026!M3:M100,$B88)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A88,Sep2026!M3:M100,$B88)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A88,Oct2026!M3:M100,$B88)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A88,Nov2026!M3:M100,$B88)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A88,Dec2026!M3:M100,$B88)</f>
         <v/>
       </c>
-      <c r="D88" s="11" t="n"/>
-      <c r="G88" s="11" t="n"/>
-      <c r="J88" s="11" t="n"/>
-      <c r="M88" s="11" t="n"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2070,7 +1916,7 @@
           <t>Buildings &amp; Amenities</t>
         </is>
       </c>
-      <c r="B89" s="11" t="inlineStr">
+      <c r="B89" t="inlineStr">
         <is>
           <t>Security Room</t>
         </is>
@@ -2079,10 +1925,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A89,Jan2026!M3:M100,$B89)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A89,Feb2026!M3:M100,$B89)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A89,Mar2026!M3:M100,$B89)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A89,Apr2026!M3:M100,$B89)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A89,May2026!M3:M100,$B89)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A89,Jun2026!M3:M100,$B89)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A89,Jul2026!M3:M100,$B89)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A89,Aug2026!M3:M100,$B89)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A89,Sep2026!M3:M100,$B89)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A89,Oct2026!M3:M100,$B89)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A89,Nov2026!M3:M100,$B89)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A89,Dec2026!M3:M100,$B89)</f>
         <v/>
       </c>
-      <c r="D89" s="11" t="n"/>
-      <c r="G89" s="11" t="n"/>
-      <c r="J89" s="11" t="n"/>
-      <c r="M89" s="11" t="n"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2090,7 +1932,7 @@
           <t>Buildings &amp; Amenities</t>
         </is>
       </c>
-      <c r="B90" s="11" t="inlineStr">
+      <c r="B90" t="inlineStr">
         <is>
           <t>Site Office</t>
         </is>
@@ -2099,10 +1941,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A90,Jan2026!M3:M100,$B90)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A90,Feb2026!M3:M100,$B90)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A90,Mar2026!M3:M100,$B90)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A90,Apr2026!M3:M100,$B90)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A90,May2026!M3:M100,$B90)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A90,Jun2026!M3:M100,$B90)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A90,Jul2026!M3:M100,$B90)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A90,Aug2026!M3:M100,$B90)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A90,Sep2026!M3:M100,$B90)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A90,Oct2026!M3:M100,$B90)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A90,Nov2026!M3:M100,$B90)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A90,Dec2026!M3:M100,$B90)</f>
         <v/>
       </c>
-      <c r="D90" s="11" t="n"/>
-      <c r="G90" s="11" t="n"/>
-      <c r="J90" s="11" t="n"/>
-      <c r="M90" s="11" t="n"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2110,7 +1948,7 @@
           <t>Buildings &amp; Amenities</t>
         </is>
       </c>
-      <c r="B91" s="11" t="inlineStr">
+      <c r="B91" t="inlineStr">
         <is>
           <t>Clubhouse</t>
         </is>
@@ -2119,10 +1957,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A91,Jan2026!M3:M100,$B91)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A91,Feb2026!M3:M100,$B91)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A91,Mar2026!M3:M100,$B91)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A91,Apr2026!M3:M100,$B91)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A91,May2026!M3:M100,$B91)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A91,Jun2026!M3:M100,$B91)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A91,Jul2026!M3:M100,$B91)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A91,Aug2026!M3:M100,$B91)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A91,Sep2026!M3:M100,$B91)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A91,Oct2026!M3:M100,$B91)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A91,Nov2026!M3:M100,$B91)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A91,Dec2026!M3:M100,$B91)</f>
         <v/>
       </c>
-      <c r="D91" s="11" t="n"/>
-      <c r="G91" s="11" t="n"/>
-      <c r="J91" s="11" t="n"/>
-      <c r="M91" s="11" t="n"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2130,7 +1964,7 @@
           <t>Buildings &amp; Amenities</t>
         </is>
       </c>
-      <c r="B92" s="11" t="inlineStr">
+      <c r="B92" t="inlineStr">
         <is>
           <t>Swimming Pool</t>
         </is>
@@ -2139,10 +1973,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A92,Jan2026!M3:M100,$B92)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A92,Feb2026!M3:M100,$B92)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A92,Mar2026!M3:M100,$B92)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A92,Apr2026!M3:M100,$B92)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A92,May2026!M3:M100,$B92)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A92,Jun2026!M3:M100,$B92)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A92,Jul2026!M3:M100,$B92)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A92,Aug2026!M3:M100,$B92)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A92,Sep2026!M3:M100,$B92)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A92,Oct2026!M3:M100,$B92)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A92,Nov2026!M3:M100,$B92)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A92,Dec2026!M3:M100,$B92)</f>
         <v/>
       </c>
-      <c r="D92" s="11" t="n"/>
-      <c r="G92" s="11" t="n"/>
-      <c r="J92" s="11" t="n"/>
-      <c r="M92" s="11" t="n"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2150,7 +1980,7 @@
           <t>Buildings &amp; Amenities</t>
         </is>
       </c>
-      <c r="B93" s="11" t="inlineStr">
+      <c r="B93" t="inlineStr">
         <is>
           <t>Gazebo</t>
         </is>
@@ -2159,10 +1989,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A93,Jan2026!M3:M100,$B93)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A93,Feb2026!M3:M100,$B93)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A93,Mar2026!M3:M100,$B93)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A93,Apr2026!M3:M100,$B93)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A93,May2026!M3:M100,$B93)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A93,Jun2026!M3:M100,$B93)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A93,Jul2026!M3:M100,$B93)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A93,Aug2026!M3:M100,$B93)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A93,Sep2026!M3:M100,$B93)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A93,Oct2026!M3:M100,$B93)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A93,Nov2026!M3:M100,$B93)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A93,Dec2026!M3:M100,$B93)</f>
         <v/>
       </c>
-      <c r="D93" s="11" t="n"/>
-      <c r="G93" s="11" t="n"/>
-      <c r="J93" s="11" t="n"/>
-      <c r="M93" s="11" t="n"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2170,7 +1996,7 @@
           <t>Buildings &amp; Amenities</t>
         </is>
       </c>
-      <c r="B94" s="11" t="inlineStr">
+      <c r="B94" t="inlineStr">
         <is>
           <t>Children's Play Area</t>
         </is>
@@ -2179,10 +2005,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A94,Jan2026!M3:M100,$B94)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A94,Feb2026!M3:M100,$B94)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A94,Mar2026!M3:M100,$B94)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A94,Apr2026!M3:M100,$B94)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A94,May2026!M3:M100,$B94)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A94,Jun2026!M3:M100,$B94)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A94,Jul2026!M3:M100,$B94)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A94,Aug2026!M3:M100,$B94)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A94,Sep2026!M3:M100,$B94)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A94,Oct2026!M3:M100,$B94)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A94,Nov2026!M3:M100,$B94)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A94,Dec2026!M3:M100,$B94)</f>
         <v/>
       </c>
-      <c r="D94" s="11" t="n"/>
-      <c r="G94" s="11" t="n"/>
-      <c r="J94" s="11" t="n"/>
-      <c r="M94" s="11" t="n"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2190,7 +2012,7 @@
           <t>Buildings &amp; Amenities</t>
         </is>
       </c>
-      <c r="B95" s="11" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>Sports Courts</t>
         </is>
@@ -2199,10 +2021,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A95,Jan2026!M3:M100,$B95)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A95,Feb2026!M3:M100,$B95)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A95,Mar2026!M3:M100,$B95)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A95,Apr2026!M3:M100,$B95)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A95,May2026!M3:M100,$B95)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A95,Jun2026!M3:M100,$B95)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A95,Jul2026!M3:M100,$B95)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A95,Aug2026!M3:M100,$B95)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A95,Sep2026!M3:M100,$B95)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A95,Oct2026!M3:M100,$B95)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A95,Nov2026!M3:M100,$B95)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A95,Dec2026!M3:M100,$B95)</f>
         <v/>
       </c>
-      <c r="D95" s="11" t="n"/>
-      <c r="G95" s="11" t="n"/>
-      <c r="J95" s="11" t="n"/>
-      <c r="M95" s="11" t="n"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2210,7 +2028,7 @@
           <t>Buildings &amp; Amenities</t>
         </is>
       </c>
-      <c r="B96" s="11" t="inlineStr">
+      <c r="B96" t="inlineStr">
         <is>
           <t>Toilets</t>
         </is>
@@ -2219,10 +2037,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A96,Jan2026!M3:M100,$B96)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A96,Feb2026!M3:M100,$B96)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A96,Mar2026!M3:M100,$B96)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A96,Apr2026!M3:M100,$B96)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A96,May2026!M3:M100,$B96)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A96,Jun2026!M3:M100,$B96)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A96,Jul2026!M3:M100,$B96)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A96,Aug2026!M3:M100,$B96)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A96,Sep2026!M3:M100,$B96)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A96,Oct2026!M3:M100,$B96)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A96,Nov2026!M3:M100,$B96)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A96,Dec2026!M3:M100,$B96)</f>
         <v/>
       </c>
-      <c r="D96" s="11" t="n"/>
-      <c r="G96" s="11" t="n"/>
-      <c r="J96" s="11" t="n"/>
-      <c r="M96" s="11" t="n"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2230,7 +2044,7 @@
           <t>Labour &amp; Contractors</t>
         </is>
       </c>
-      <c r="B97" s="11" t="inlineStr">
+      <c r="B97" t="inlineStr">
         <is>
           <t>Labour Wages</t>
         </is>
@@ -2239,10 +2053,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A97,Jan2026!M3:M100,$B97)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A97,Feb2026!M3:M100,$B97)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A97,Mar2026!M3:M100,$B97)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A97,Apr2026!M3:M100,$B97)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A97,May2026!M3:M100,$B97)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A97,Jun2026!M3:M100,$B97)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A97,Jul2026!M3:M100,$B97)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A97,Aug2026!M3:M100,$B97)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A97,Sep2026!M3:M100,$B97)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A97,Oct2026!M3:M100,$B97)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A97,Nov2026!M3:M100,$B97)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A97,Dec2026!M3:M100,$B97)</f>
         <v/>
       </c>
-      <c r="D97" s="11" t="n"/>
-      <c r="G97" s="11" t="n"/>
-      <c r="J97" s="11" t="n"/>
-      <c r="M97" s="11" t="n"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2250,7 +2060,7 @@
           <t>Labour &amp; Contractors</t>
         </is>
       </c>
-      <c r="B98" s="11" t="inlineStr">
+      <c r="B98" t="inlineStr">
         <is>
           <t>Contractor Payments</t>
         </is>
@@ -2259,10 +2069,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A98,Jan2026!M3:M100,$B98)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A98,Feb2026!M3:M100,$B98)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A98,Mar2026!M3:M100,$B98)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A98,Apr2026!M3:M100,$B98)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A98,May2026!M3:M100,$B98)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A98,Jun2026!M3:M100,$B98)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A98,Jul2026!M3:M100,$B98)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A98,Aug2026!M3:M100,$B98)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A98,Sep2026!M3:M100,$B98)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A98,Oct2026!M3:M100,$B98)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A98,Nov2026!M3:M100,$B98)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A98,Dec2026!M3:M100,$B98)</f>
         <v/>
       </c>
-      <c r="D98" s="11" t="n"/>
-      <c r="G98" s="11" t="n"/>
-      <c r="J98" s="11" t="n"/>
-      <c r="M98" s="11" t="n"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2270,7 +2076,7 @@
           <t>Labour &amp; Contractors</t>
         </is>
       </c>
-      <c r="B99" s="11" t="inlineStr">
+      <c r="B99" t="inlineStr">
         <is>
           <t>Machinery Hire</t>
         </is>
@@ -2279,10 +2085,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A99,Jan2026!M3:M100,$B99)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A99,Feb2026!M3:M100,$B99)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A99,Mar2026!M3:M100,$B99)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A99,Apr2026!M3:M100,$B99)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A99,May2026!M3:M100,$B99)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A99,Jun2026!M3:M100,$B99)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A99,Jul2026!M3:M100,$B99)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A99,Aug2026!M3:M100,$B99)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A99,Sep2026!M3:M100,$B99)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A99,Oct2026!M3:M100,$B99)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A99,Nov2026!M3:M100,$B99)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A99,Dec2026!M3:M100,$B99)</f>
         <v/>
       </c>
-      <c r="D99" s="11" t="n"/>
-      <c r="G99" s="11" t="n"/>
-      <c r="J99" s="11" t="n"/>
-      <c r="M99" s="11" t="n"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2290,7 +2092,7 @@
           <t>Labour &amp; Contractors</t>
         </is>
       </c>
-      <c r="B100" s="11" t="inlineStr">
+      <c r="B100" t="inlineStr">
         <is>
           <t>Excavator/JCB</t>
         </is>
@@ -2299,10 +2101,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A100,Jan2026!M3:M100,$B100)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A100,Feb2026!M3:M100,$B100)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A100,Mar2026!M3:M100,$B100)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A100,Apr2026!M3:M100,$B100)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A100,May2026!M3:M100,$B100)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A100,Jun2026!M3:M100,$B100)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A100,Jul2026!M3:M100,$B100)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A100,Aug2026!M3:M100,$B100)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A100,Sep2026!M3:M100,$B100)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A100,Oct2026!M3:M100,$B100)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A100,Nov2026!M3:M100,$B100)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A100,Dec2026!M3:M100,$B100)</f>
         <v/>
       </c>
-      <c r="D100" s="11" t="n"/>
-      <c r="G100" s="11" t="n"/>
-      <c r="J100" s="11" t="n"/>
-      <c r="M100" s="11" t="n"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2310,7 +2108,7 @@
           <t>Labour &amp; Contractors</t>
         </is>
       </c>
-      <c r="B101" s="11" t="inlineStr">
+      <c r="B101" t="inlineStr">
         <is>
           <t>Tractor &amp; Transport</t>
         </is>
@@ -2319,10 +2117,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A101,Jan2026!M3:M100,$B101)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A101,Feb2026!M3:M100,$B101)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A101,Mar2026!M3:M100,$B101)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A101,Apr2026!M3:M100,$B101)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A101,May2026!M3:M100,$B101)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A101,Jun2026!M3:M100,$B101)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A101,Jul2026!M3:M100,$B101)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A101,Aug2026!M3:M100,$B101)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A101,Sep2026!M3:M100,$B101)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A101,Oct2026!M3:M100,$B101)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A101,Nov2026!M3:M100,$B101)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A101,Dec2026!M3:M100,$B101)</f>
         <v/>
       </c>
-      <c r="D101" s="11" t="n"/>
-      <c r="G101" s="11" t="n"/>
-      <c r="J101" s="11" t="n"/>
-      <c r="M101" s="11" t="n"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2330,7 +2124,7 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="B102" s="11" t="inlineStr">
+      <c r="B102" t="inlineStr">
         <is>
           <t>Cement</t>
         </is>
@@ -2339,10 +2133,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A102,Jan2026!M3:M100,$B102)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A102,Feb2026!M3:M100,$B102)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A102,Mar2026!M3:M100,$B102)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A102,Apr2026!M3:M100,$B102)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A102,May2026!M3:M100,$B102)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A102,Jun2026!M3:M100,$B102)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A102,Jul2026!M3:M100,$B102)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A102,Aug2026!M3:M100,$B102)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A102,Sep2026!M3:M100,$B102)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A102,Oct2026!M3:M100,$B102)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A102,Nov2026!M3:M100,$B102)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A102,Dec2026!M3:M100,$B102)</f>
         <v/>
       </c>
-      <c r="D102" s="11" t="n"/>
-      <c r="G102" s="11" t="n"/>
-      <c r="J102" s="11" t="n"/>
-      <c r="M102" s="11" t="n"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2350,7 +2140,7 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="B103" s="11" t="inlineStr">
+      <c r="B103" t="inlineStr">
         <is>
           <t>Sand</t>
         </is>
@@ -2359,10 +2149,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A103,Jan2026!M3:M100,$B103)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A103,Feb2026!M3:M100,$B103)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A103,Mar2026!M3:M100,$B103)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A103,Apr2026!M3:M100,$B103)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A103,May2026!M3:M100,$B103)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A103,Jun2026!M3:M100,$B103)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A103,Jul2026!M3:M100,$B103)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A103,Aug2026!M3:M100,$B103)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A103,Sep2026!M3:M100,$B103)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A103,Oct2026!M3:M100,$B103)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A103,Nov2026!M3:M100,$B103)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A103,Dec2026!M3:M100,$B103)</f>
         <v/>
       </c>
-      <c r="D103" s="11" t="n"/>
-      <c r="G103" s="11" t="n"/>
-      <c r="J103" s="11" t="n"/>
-      <c r="M103" s="11" t="n"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2370,7 +2156,7 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="B104" s="11" t="inlineStr">
+      <c r="B104" t="inlineStr">
         <is>
           <t>Metal</t>
         </is>
@@ -2379,10 +2165,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A104,Jan2026!M3:M100,$B104)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A104,Feb2026!M3:M100,$B104)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A104,Mar2026!M3:M100,$B104)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A104,Apr2026!M3:M100,$B104)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A104,May2026!M3:M100,$B104)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A104,Jun2026!M3:M100,$B104)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A104,Jul2026!M3:M100,$B104)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A104,Aug2026!M3:M100,$B104)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A104,Sep2026!M3:M100,$B104)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A104,Oct2026!M3:M100,$B104)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A104,Nov2026!M3:M100,$B104)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A104,Dec2026!M3:M100,$B104)</f>
         <v/>
       </c>
-      <c r="D104" s="11" t="n"/>
-      <c r="G104" s="11" t="n"/>
-      <c r="J104" s="11" t="n"/>
-      <c r="M104" s="11" t="n"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2390,7 +2172,7 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="B105" s="11" t="inlineStr">
+      <c r="B105" t="inlineStr">
         <is>
           <t>Bricks</t>
         </is>
@@ -2399,10 +2181,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A105,Jan2026!M3:M100,$B105)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A105,Feb2026!M3:M100,$B105)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A105,Mar2026!M3:M100,$B105)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A105,Apr2026!M3:M100,$B105)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A105,May2026!M3:M100,$B105)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A105,Jun2026!M3:M100,$B105)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A105,Jul2026!M3:M100,$B105)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A105,Aug2026!M3:M100,$B105)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A105,Sep2026!M3:M100,$B105)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A105,Oct2026!M3:M100,$B105)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A105,Nov2026!M3:M100,$B105)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A105,Dec2026!M3:M100,$B105)</f>
         <v/>
       </c>
-      <c r="D105" s="11" t="n"/>
-      <c r="G105" s="11" t="n"/>
-      <c r="J105" s="11" t="n"/>
-      <c r="M105" s="11" t="n"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2410,7 +2188,7 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="B106" s="11" t="inlineStr">
+      <c r="B106" t="inlineStr">
         <is>
           <t>Steel</t>
         </is>
@@ -2419,10 +2197,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A106,Jan2026!M3:M100,$B106)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A106,Feb2026!M3:M100,$B106)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A106,Mar2026!M3:M100,$B106)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A106,Apr2026!M3:M100,$B106)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A106,May2026!M3:M100,$B106)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A106,Jun2026!M3:M100,$B106)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A106,Jul2026!M3:M100,$B106)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A106,Aug2026!M3:M100,$B106)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A106,Sep2026!M3:M100,$B106)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A106,Oct2026!M3:M100,$B106)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A106,Nov2026!M3:M100,$B106)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A106,Dec2026!M3:M100,$B106)</f>
         <v/>
       </c>
-      <c r="D106" s="11" t="n"/>
-      <c r="G106" s="11" t="n"/>
-      <c r="J106" s="11" t="n"/>
-      <c r="M106" s="11" t="n"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2430,7 +2204,7 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="B107" s="11" t="inlineStr">
+      <c r="B107" t="inlineStr">
         <is>
           <t>Pipes</t>
         </is>
@@ -2439,10 +2213,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A107,Jan2026!M3:M100,$B107)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A107,Feb2026!M3:M100,$B107)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A107,Mar2026!M3:M100,$B107)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A107,Apr2026!M3:M100,$B107)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A107,May2026!M3:M100,$B107)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A107,Jun2026!M3:M100,$B107)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A107,Jul2026!M3:M100,$B107)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A107,Aug2026!M3:M100,$B107)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A107,Sep2026!M3:M100,$B107)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A107,Oct2026!M3:M100,$B107)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A107,Nov2026!M3:M100,$B107)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A107,Dec2026!M3:M100,$B107)</f>
         <v/>
       </c>
-      <c r="D107" s="11" t="n"/>
-      <c r="G107" s="11" t="n"/>
-      <c r="J107" s="11" t="n"/>
-      <c r="M107" s="11" t="n"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2450,7 +2220,7 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="B108" s="11" t="inlineStr">
+      <c r="B108" t="inlineStr">
         <is>
           <t>Electrical Materials</t>
         </is>
@@ -2459,10 +2229,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A108,Jan2026!M3:M100,$B108)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A108,Feb2026!M3:M100,$B108)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A108,Mar2026!M3:M100,$B108)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A108,Apr2026!M3:M100,$B108)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A108,May2026!M3:M100,$B108)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A108,Jun2026!M3:M100,$B108)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A108,Jul2026!M3:M100,$B108)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A108,Aug2026!M3:M100,$B108)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A108,Sep2026!M3:M100,$B108)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A108,Oct2026!M3:M100,$B108)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A108,Nov2026!M3:M100,$B108)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A108,Dec2026!M3:M100,$B108)</f>
         <v/>
       </c>
-      <c r="D108" s="11" t="n"/>
-      <c r="G108" s="11" t="n"/>
-      <c r="J108" s="11" t="n"/>
-      <c r="M108" s="11" t="n"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2470,7 +2236,7 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="B109" s="11" t="inlineStr">
+      <c r="B109" t="inlineStr">
         <is>
           <t>Paint</t>
         </is>
@@ -2479,10 +2245,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A109,Jan2026!M3:M100,$B109)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A109,Feb2026!M3:M100,$B109)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A109,Mar2026!M3:M100,$B109)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A109,Apr2026!M3:M100,$B109)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A109,May2026!M3:M100,$B109)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A109,Jun2026!M3:M100,$B109)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A109,Jul2026!M3:M100,$B109)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A109,Aug2026!M3:M100,$B109)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A109,Sep2026!M3:M100,$B109)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A109,Oct2026!M3:M100,$B109)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A109,Nov2026!M3:M100,$B109)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A109,Dec2026!M3:M100,$B109)</f>
         <v/>
       </c>
-      <c r="D109" s="11" t="n"/>
-      <c r="G109" s="11" t="n"/>
-      <c r="J109" s="11" t="n"/>
-      <c r="M109" s="11" t="n"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2490,7 +2252,7 @@
           <t>Materials</t>
         </is>
       </c>
-      <c r="B110" s="11" t="inlineStr">
+      <c r="B110" t="inlineStr">
         <is>
           <t>Tiles</t>
         </is>
@@ -2499,10 +2261,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A110,Jan2026!M3:M100,$B110)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A110,Feb2026!M3:M100,$B110)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A110,Mar2026!M3:M100,$B110)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A110,Apr2026!M3:M100,$B110)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A110,May2026!M3:M100,$B110)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A110,Jun2026!M3:M100,$B110)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A110,Jul2026!M3:M100,$B110)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A110,Aug2026!M3:M100,$B110)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A110,Sep2026!M3:M100,$B110)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A110,Oct2026!M3:M100,$B110)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A110,Nov2026!M3:M100,$B110)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A110,Dec2026!M3:M100,$B110)</f>
         <v/>
       </c>
-      <c r="D110" s="11" t="n"/>
-      <c r="G110" s="11" t="n"/>
-      <c r="J110" s="11" t="n"/>
-      <c r="M110" s="11" t="n"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2510,7 +2268,7 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="B111" s="11" t="inlineStr">
+      <c r="B111" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
@@ -2519,10 +2277,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A111,Jan2026!M3:M100,$B111)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A111,Feb2026!M3:M100,$B111)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A111,Mar2026!M3:M100,$B111)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A111,Apr2026!M3:M100,$B111)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A111,May2026!M3:M100,$B111)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A111,Jun2026!M3:M100,$B111)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A111,Jul2026!M3:M100,$B111)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A111,Aug2026!M3:M100,$B111)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A111,Sep2026!M3:M100,$B111)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A111,Oct2026!M3:M100,$B111)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A111,Nov2026!M3:M100,$B111)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A111,Dec2026!M3:M100,$B111)</f>
         <v/>
       </c>
-      <c r="D111" s="11" t="n"/>
-      <c r="G111" s="11" t="n"/>
-      <c r="J111" s="11" t="n"/>
-      <c r="M111" s="11" t="n"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2530,7 +2284,7 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="B112" s="11" t="inlineStr">
+      <c r="B112" t="inlineStr">
         <is>
           <t>Housekeeping</t>
         </is>
@@ -2539,10 +2293,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A112,Jan2026!M3:M100,$B112)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A112,Feb2026!M3:M100,$B112)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A112,Mar2026!M3:M100,$B112)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A112,Apr2026!M3:M100,$B112)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A112,May2026!M3:M100,$B112)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A112,Jun2026!M3:M100,$B112)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A112,Jul2026!M3:M100,$B112)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A112,Aug2026!M3:M100,$B112)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A112,Sep2026!M3:M100,$B112)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A112,Oct2026!M3:M100,$B112)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A112,Nov2026!M3:M100,$B112)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A112,Dec2026!M3:M100,$B112)</f>
         <v/>
       </c>
-      <c r="D112" s="11" t="n"/>
-      <c r="G112" s="11" t="n"/>
-      <c r="J112" s="11" t="n"/>
-      <c r="M112" s="11" t="n"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2550,7 +2300,7 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="B113" s="11" t="inlineStr">
+      <c r="B113" t="inlineStr">
         <is>
           <t>Fuel &amp; Diesel</t>
         </is>
@@ -2559,10 +2309,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A113,Jan2026!M3:M100,$B113)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A113,Feb2026!M3:M100,$B113)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A113,Mar2026!M3:M100,$B113)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A113,Apr2026!M3:M100,$B113)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A113,May2026!M3:M100,$B113)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A113,Jun2026!M3:M100,$B113)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A113,Jul2026!M3:M100,$B113)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A113,Aug2026!M3:M100,$B113)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A113,Sep2026!M3:M100,$B113)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A113,Oct2026!M3:M100,$B113)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A113,Nov2026!M3:M100,$B113)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A113,Dec2026!M3:M100,$B113)</f>
         <v/>
       </c>
-      <c r="D113" s="11" t="n"/>
-      <c r="G113" s="11" t="n"/>
-      <c r="J113" s="11" t="n"/>
-      <c r="M113" s="11" t="n"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2570,7 +2316,7 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="B114" s="11" t="inlineStr">
+      <c r="B114" t="inlineStr">
         <is>
           <t>Vehicle Expenses</t>
         </is>
@@ -2579,10 +2325,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A114,Jan2026!M3:M100,$B114)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A114,Feb2026!M3:M100,$B114)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A114,Mar2026!M3:M100,$B114)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A114,Apr2026!M3:M100,$B114)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A114,May2026!M3:M100,$B114)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A114,Jun2026!M3:M100,$B114)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A114,Jul2026!M3:M100,$B114)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A114,Aug2026!M3:M100,$B114)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A114,Sep2026!M3:M100,$B114)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A114,Oct2026!M3:M100,$B114)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A114,Nov2026!M3:M100,$B114)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A114,Dec2026!M3:M100,$B114)</f>
         <v/>
       </c>
-      <c r="D114" s="11" t="n"/>
-      <c r="G114" s="11" t="n"/>
-      <c r="J114" s="11" t="n"/>
-      <c r="M114" s="11" t="n"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2590,7 +2332,7 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="B115" s="11" t="inlineStr">
+      <c r="B115" t="inlineStr">
         <is>
           <t>Repairs &amp; Maintenance</t>
         </is>
@@ -2599,10 +2341,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A115,Jan2026!M3:M100,$B115)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A115,Feb2026!M3:M100,$B115)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A115,Mar2026!M3:M100,$B115)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A115,Apr2026!M3:M100,$B115)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A115,May2026!M3:M100,$B115)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A115,Jun2026!M3:M100,$B115)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A115,Jul2026!M3:M100,$B115)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A115,Aug2026!M3:M100,$B115)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A115,Sep2026!M3:M100,$B115)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A115,Oct2026!M3:M100,$B115)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A115,Nov2026!M3:M100,$B115)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A115,Dec2026!M3:M100,$B115)</f>
         <v/>
       </c>
-      <c r="D115" s="11" t="n"/>
-      <c r="G115" s="11" t="n"/>
-      <c r="J115" s="11" t="n"/>
-      <c r="M115" s="11" t="n"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2610,7 +2348,7 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="B116" s="11" t="inlineStr">
+      <c r="B116" t="inlineStr">
         <is>
           <t>Office Expenses</t>
         </is>
@@ -2619,10 +2357,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A116,Jan2026!M3:M100,$B116)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A116,Feb2026!M3:M100,$B116)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A116,Mar2026!M3:M100,$B116)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A116,Apr2026!M3:M100,$B116)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A116,May2026!M3:M100,$B116)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A116,Jun2026!M3:M100,$B116)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A116,Jul2026!M3:M100,$B116)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A116,Aug2026!M3:M100,$B116)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A116,Sep2026!M3:M100,$B116)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A116,Oct2026!M3:M100,$B116)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A116,Nov2026!M3:M100,$B116)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A116,Dec2026!M3:M100,$B116)</f>
         <v/>
       </c>
-      <c r="D116" s="11" t="n"/>
-      <c r="G116" s="11" t="n"/>
-      <c r="J116" s="11" t="n"/>
-      <c r="M116" s="11" t="n"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2630,7 +2364,7 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="B117" s="11" t="inlineStr">
+      <c r="B117" t="inlineStr">
         <is>
           <t>Internet &amp; Phone</t>
         </is>
@@ -2639,10 +2373,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A117,Jan2026!M3:M100,$B117)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A117,Feb2026!M3:M100,$B117)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A117,Mar2026!M3:M100,$B117)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A117,Apr2026!M3:M100,$B117)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A117,May2026!M3:M100,$B117)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A117,Jun2026!M3:M100,$B117)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A117,Jul2026!M3:M100,$B117)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A117,Aug2026!M3:M100,$B117)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A117,Sep2026!M3:M100,$B117)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A117,Oct2026!M3:M100,$B117)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A117,Nov2026!M3:M100,$B117)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A117,Dec2026!M3:M100,$B117)</f>
         <v/>
       </c>
-      <c r="D117" s="11" t="n"/>
-      <c r="G117" s="11" t="n"/>
-      <c r="J117" s="11" t="n"/>
-      <c r="M117" s="11" t="n"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -2650,7 +2380,7 @@
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B118" s="11" t="inlineStr">
+      <c r="B118" t="inlineStr">
         <is>
           <t>Advertisement</t>
         </is>
@@ -2659,10 +2389,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A118,Jan2026!M3:M100,$B118)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A118,Feb2026!M3:M100,$B118)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A118,Mar2026!M3:M100,$B118)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A118,Apr2026!M3:M100,$B118)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A118,May2026!M3:M100,$B118)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A118,Jun2026!M3:M100,$B118)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A118,Jul2026!M3:M100,$B118)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A118,Aug2026!M3:M100,$B118)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A118,Sep2026!M3:M100,$B118)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A118,Oct2026!M3:M100,$B118)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A118,Nov2026!M3:M100,$B118)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A118,Dec2026!M3:M100,$B118)</f>
         <v/>
       </c>
-      <c r="D118" s="11" t="n"/>
-      <c r="G118" s="11" t="n"/>
-      <c r="J118" s="11" t="n"/>
-      <c r="M118" s="11" t="n"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2670,7 +2396,7 @@
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B119" s="11" t="inlineStr">
+      <c r="B119" t="inlineStr">
         <is>
           <t>Flex Boards</t>
         </is>
@@ -2679,10 +2405,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A119,Jan2026!M3:M100,$B119)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A119,Feb2026!M3:M100,$B119)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A119,Mar2026!M3:M100,$B119)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A119,Apr2026!M3:M100,$B119)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A119,May2026!M3:M100,$B119)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A119,Jun2026!M3:M100,$B119)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A119,Jul2026!M3:M100,$B119)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A119,Aug2026!M3:M100,$B119)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A119,Sep2026!M3:M100,$B119)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A119,Oct2026!M3:M100,$B119)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A119,Nov2026!M3:M100,$B119)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A119,Dec2026!M3:M100,$B119)</f>
         <v/>
       </c>
-      <c r="D119" s="11" t="n"/>
-      <c r="G119" s="11" t="n"/>
-      <c r="J119" s="11" t="n"/>
-      <c r="M119" s="11" t="n"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2690,7 +2412,7 @@
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B120" s="11" t="inlineStr">
+      <c r="B120" t="inlineStr">
         <is>
           <t>Brochures</t>
         </is>
@@ -2699,10 +2421,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A120,Jan2026!M3:M100,$B120)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A120,Feb2026!M3:M100,$B120)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A120,Mar2026!M3:M100,$B120)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A120,Apr2026!M3:M100,$B120)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A120,May2026!M3:M100,$B120)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A120,Jun2026!M3:M100,$B120)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A120,Jul2026!M3:M100,$B120)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A120,Aug2026!M3:M100,$B120)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A120,Sep2026!M3:M100,$B120)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A120,Oct2026!M3:M100,$B120)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A120,Nov2026!M3:M100,$B120)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A120,Dec2026!M3:M100,$B120)</f>
         <v/>
       </c>
-      <c r="D120" s="11" t="n"/>
-      <c r="G120" s="11" t="n"/>
-      <c r="J120" s="11" t="n"/>
-      <c r="M120" s="11" t="n"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2710,7 +2428,7 @@
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B121" s="11" t="inlineStr">
+      <c r="B121" t="inlineStr">
         <is>
           <t>Events</t>
         </is>
@@ -2719,10 +2437,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A121,Jan2026!M3:M100,$B121)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A121,Feb2026!M3:M100,$B121)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A121,Mar2026!M3:M100,$B121)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A121,Apr2026!M3:M100,$B121)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A121,May2026!M3:M100,$B121)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A121,Jun2026!M3:M100,$B121)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A121,Jul2026!M3:M100,$B121)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A121,Aug2026!M3:M100,$B121)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A121,Sep2026!M3:M100,$B121)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A121,Oct2026!M3:M100,$B121)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A121,Nov2026!M3:M100,$B121)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A121,Dec2026!M3:M100,$B121)</f>
         <v/>
       </c>
-      <c r="D121" s="11" t="n"/>
-      <c r="G121" s="11" t="n"/>
-      <c r="J121" s="11" t="n"/>
-      <c r="M121" s="11" t="n"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2730,7 +2444,7 @@
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B122" s="11" t="inlineStr">
+      <c r="B122" t="inlineStr">
         <is>
           <t>Photography &amp; Drone</t>
         </is>
@@ -2739,10 +2453,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A122,Jan2026!M3:M100,$B122)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A122,Feb2026!M3:M100,$B122)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A122,Mar2026!M3:M100,$B122)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A122,Apr2026!M3:M100,$B122)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A122,May2026!M3:M100,$B122)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A122,Jun2026!M3:M100,$B122)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A122,Jul2026!M3:M100,$B122)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A122,Aug2026!M3:M100,$B122)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A122,Sep2026!M3:M100,$B122)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A122,Oct2026!M3:M100,$B122)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A122,Nov2026!M3:M100,$B122)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A122,Dec2026!M3:M100,$B122)</f>
         <v/>
       </c>
-      <c r="D122" s="11" t="n"/>
-      <c r="G122" s="11" t="n"/>
-      <c r="J122" s="11" t="n"/>
-      <c r="M122" s="11" t="n"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -2750,7 +2460,7 @@
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B123" s="11" t="inlineStr">
+      <c r="B123" t="inlineStr">
         <is>
           <t>Digital Marketing</t>
         </is>
@@ -2759,10 +2469,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A123,Jan2026!M3:M100,$B123)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A123,Feb2026!M3:M100,$B123)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A123,Mar2026!M3:M100,$B123)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A123,Apr2026!M3:M100,$B123)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A123,May2026!M3:M100,$B123)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A123,Jun2026!M3:M100,$B123)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A123,Jul2026!M3:M100,$B123)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A123,Aug2026!M3:M100,$B123)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A123,Sep2026!M3:M100,$B123)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A123,Oct2026!M3:M100,$B123)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A123,Nov2026!M3:M100,$B123)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A123,Dec2026!M3:M100,$B123)</f>
         <v/>
       </c>
-      <c r="D123" s="11" t="n"/>
-      <c r="G123" s="11" t="n"/>
-      <c r="J123" s="11" t="n"/>
-      <c r="M123" s="11" t="n"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -2770,7 +2476,7 @@
           <t>Miscellaneous</t>
         </is>
       </c>
-      <c r="B124" s="11" t="inlineStr">
+      <c r="B124" t="inlineStr">
         <is>
           <t>Travel Expenses</t>
         </is>
@@ -2779,10 +2485,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A124,Jan2026!M3:M100,$B124)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A124,Feb2026!M3:M100,$B124)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A124,Mar2026!M3:M100,$B124)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A124,Apr2026!M3:M100,$B124)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A124,May2026!M3:M100,$B124)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A124,Jun2026!M3:M100,$B124)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A124,Jul2026!M3:M100,$B124)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A124,Aug2026!M3:M100,$B124)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A124,Sep2026!M3:M100,$B124)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A124,Oct2026!M3:M100,$B124)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A124,Nov2026!M3:M100,$B124)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A124,Dec2026!M3:M100,$B124)</f>
         <v/>
       </c>
-      <c r="D124" s="11" t="n"/>
-      <c r="G124" s="11" t="n"/>
-      <c r="J124" s="11" t="n"/>
-      <c r="M124" s="11" t="n"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2790,7 +2492,7 @@
           <t>Miscellaneous</t>
         </is>
       </c>
-      <c r="B125" s="11" t="inlineStr">
+      <c r="B125" t="inlineStr">
         <is>
           <t>Food &amp; Refreshments</t>
         </is>
@@ -2799,10 +2501,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A125,Jan2026!M3:M100,$B125)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A125,Feb2026!M3:M100,$B125)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A125,Mar2026!M3:M100,$B125)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A125,Apr2026!M3:M100,$B125)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A125,May2026!M3:M100,$B125)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A125,Jun2026!M3:M100,$B125)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A125,Jul2026!M3:M100,$B125)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A125,Aug2026!M3:M100,$B125)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A125,Sep2026!M3:M100,$B125)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A125,Oct2026!M3:M100,$B125)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A125,Nov2026!M3:M100,$B125)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A125,Dec2026!M3:M100,$B125)</f>
         <v/>
       </c>
-      <c r="D125" s="11" t="n"/>
-      <c r="G125" s="11" t="n"/>
-      <c r="J125" s="11" t="n"/>
-      <c r="M125" s="11" t="n"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -2810,7 +2508,7 @@
           <t>Miscellaneous</t>
         </is>
       </c>
-      <c r="B126" s="11" t="inlineStr">
+      <c r="B126" t="inlineStr">
         <is>
           <t>Government Fees</t>
         </is>
@@ -2819,10 +2517,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A126,Jan2026!M3:M100,$B126)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A126,Feb2026!M3:M100,$B126)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A126,Mar2026!M3:M100,$B126)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A126,Apr2026!M3:M100,$B126)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A126,May2026!M3:M100,$B126)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A126,Jun2026!M3:M100,$B126)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A126,Jul2026!M3:M100,$B126)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A126,Aug2026!M3:M100,$B126)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A126,Sep2026!M3:M100,$B126)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A126,Oct2026!M3:M100,$B126)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A126,Nov2026!M3:M100,$B126)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A126,Dec2026!M3:M100,$B126)</f>
         <v/>
       </c>
-      <c r="D126" s="11" t="n"/>
-      <c r="G126" s="11" t="n"/>
-      <c r="J126" s="11" t="n"/>
-      <c r="M126" s="11" t="n"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -2830,7 +2524,7 @@
           <t>Miscellaneous</t>
         </is>
       </c>
-      <c r="B127" s="11" t="inlineStr">
+      <c r="B127" t="inlineStr">
         <is>
           <t>Bank Charges</t>
         </is>
@@ -2839,10 +2533,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A127,Jan2026!M3:M100,$B127)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A127,Feb2026!M3:M100,$B127)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A127,Mar2026!M3:M100,$B127)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A127,Apr2026!M3:M100,$B127)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A127,May2026!M3:M100,$B127)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A127,Jun2026!M3:M100,$B127)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A127,Jul2026!M3:M100,$B127)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A127,Aug2026!M3:M100,$B127)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A127,Sep2026!M3:M100,$B127)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A127,Oct2026!M3:M100,$B127)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A127,Nov2026!M3:M100,$B127)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A127,Dec2026!M3:M100,$B127)</f>
         <v/>
       </c>
-      <c r="D127" s="11" t="n"/>
-      <c r="G127" s="11" t="n"/>
-      <c r="J127" s="11" t="n"/>
-      <c r="M127" s="11" t="n"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -2850,7 +2540,7 @@
           <t>Miscellaneous</t>
         </is>
       </c>
-      <c r="B128" s="11" t="inlineStr">
+      <c r="B128" t="inlineStr">
         <is>
           <t>Miscellaneous Expenses</t>
         </is>
@@ -2859,10 +2549,6 @@
         <f>SUMIFS(Jan2026!K3:K100,Jan2026!L3:L100,$A128,Jan2026!M3:M100,$B128)+SUMIFS(Feb2026!K3:K100,Feb2026!L3:L100,$A128,Feb2026!M3:M100,$B128)+SUMIFS(Mar2026!K3:K100,Mar2026!L3:L100,$A128,Mar2026!M3:M100,$B128)+SUMIFS(Apr2026!K3:K100,Apr2026!L3:L100,$A128,Apr2026!M3:M100,$B128)+SUMIFS(May2026!K3:K100,May2026!L3:L100,$A128,May2026!M3:M100,$B128)+SUMIFS(Jun2026!K3:K100,Jun2026!L3:L100,$A128,Jun2026!M3:M100,$B128)+SUMIFS(Jul2026!K3:K100,Jul2026!L3:L100,$A128,Jul2026!M3:M100,$B128)+SUMIFS(Aug2026!K3:K100,Aug2026!L3:L100,$A128,Aug2026!M3:M100,$B128)+SUMIFS(Sep2026!K3:K100,Sep2026!L3:L100,$A128,Sep2026!M3:M100,$B128)+SUMIFS(Oct2026!K3:K100,Oct2026!L3:L100,$A128,Oct2026!M3:M100,$B128)+SUMIFS(Nov2026!K3:K100,Nov2026!L3:L100,$A128,Nov2026!M3:M100,$B128)+SUMIFS(Dec2026!K3:K100,Dec2026!L3:L100,$A128,Dec2026!M3:M100,$B128)</f>
         <v/>
       </c>
-      <c r="D128" s="11" t="n"/>
-      <c r="G128" s="11" t="n"/>
-      <c r="J128" s="11" t="n"/>
-      <c r="M128" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add sample demo transactions, Dashboard print area, and PDF export macro source
- Sample Jan-May 2026 Receipts/Payments rows to demonstrate the Dashboard with real data
- Print area, landscape orientation, and fit-to-width set on Dashboard sheet for clean PDF export
- VBA macro source for a one-click Dashboard-to-PDF export button (manual setup required in Excel, see scripts/ExportDashboardToPDF.bas)
</commit_message>
<xml_diff>
--- a/expense_tracker_2026.xlsx
+++ b/expense_tracker_2026.xlsx
@@ -35,6 +35,7 @@
     <definedName name="Cat_Operations">'Categories'!$O$3:$O$9</definedName>
     <definedName name="Cat_Marketing_Sales">'Categories'!$P$3:$P$8</definedName>
     <definedName name="Cat_Miscellaneous">'Categories'!$Q$3:$Q$7</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Dashboard'!$A$1:$R$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -42,7 +43,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <name val="Calibri"/>
@@ -129,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -156,6 +159,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -957,7 +961,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -2552,6 +2556,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
@@ -3273,7 +3278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:Q70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4718,6 +4723,115 @@
       <c r="O2" s="3" t="inlineStr">
         <is>
           <t>Comments</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="14" t="n">
+        <v>46027</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Land purchase advance from investor</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Investor Capital</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="I3" s="14" t="n">
+        <v>46032</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Land purchase payment</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Land &amp; Legal</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Land Purchase</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Initial land purchase</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="14" t="n">
+        <v>46037</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Partner contribution</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Partner Contribution</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="n">
+        <v>46042</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Survey charges</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>25000</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Land &amp; Legal</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Survey Charges</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Cash</t>
         </is>
       </c>
     </row>
@@ -4897,6 +5011,86 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="14" t="n">
+        <v>46058</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Bank loan disbursement</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Loan Received</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="I3" s="14" t="n">
+        <v>46061</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Earthwork and levelling</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>300000</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Site Development</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Earthwork &amp; Levelling</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="I4" s="14" t="n">
+        <v>46071</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Labour wages</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>80000</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Labour &amp; Contractors</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Labour Wages</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+    </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
@@ -5074,6 +5268,114 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="14" t="n">
+        <v>46091</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Plot sale - Plot 12</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="I3" s="14" t="n">
+        <v>46086</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Cement purchase</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>150000</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Cement</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="I4" s="14" t="n">
+        <v>46096</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Borewell drilling</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>200000</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Borewell</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="I5" s="14" t="n">
+        <v>46106</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Advertisement</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Advertisement</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+    </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
@@ -5251,6 +5553,110 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="14" t="n">
+        <v>46117</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Plot sale - Plot 15</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="I3" s="14" t="n">
+        <v>46120</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Compound wall construction</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>350000</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Site Development</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Compound Wall</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="14" t="n">
+        <v>46132</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Partner contribution</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>300000</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Partner Contribution</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="n">
+        <v>46130</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Security guard salary</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>45000</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+    </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
@@ -5428,6 +5834,34 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="I3" s="14" t="n">
+        <v>46152</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Office expenses</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>15000</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Office Expenses</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+    </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>

</xml_diff>